<commit_message>
Validated report update 2025-11-04 14:09
</commit_message>
<xml_diff>
--- a/flagged_segments.xlsx
+++ b/flagged_segments.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="10">
   <si>
     <t>Session</t>
   </si>
@@ -28,37 +28,19 @@
     <t>Category</t>
   </si>
   <si>
-    <t>GMT20251026-075624</t>
-  </si>
-  <si>
     <t>GMT20250821-130122</t>
   </si>
   <si>
-    <t>I mean, on Tuesday, so…</t>
-  </si>
-  <si>
-    <t>Yes, it can often fix it.</t>
-  </si>
-  <si>
     <t>Oh my god, I'm so sorry, I don't know why. Some meeting rooms… in some meeting rooms in my department, the connection is weird. If I start lagging at any point, let me know again. But yeah, we lost, like.</t>
   </si>
   <si>
-    <t>Hello?</t>
-  </si>
-  <si>
-    <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20251026-075624_validated_report.html</t>
+    <t>ask them not to charge you for this class, and then I can give you a full makeup class, instead of this one, because it's unfair to just have you not understand half the things I'm saying.</t>
   </si>
   <si>
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20250821-130122_validated_report.html</t>
   </si>
   <si>
-    <t>Student Behavior Issues: Homework Non-Completion</t>
-  </si>
-  <si>
-    <t>Session Quality: Lack of Engagement</t>
-  </si>
-  <si>
-    <t>Session Quality: Session Quality</t>
+    <t>Tutor Policy Breach: Payment Outside Platform</t>
   </si>
   <si>
     <t>View Report</t>
@@ -428,7 +410,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -456,13 +438,13 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -470,49 +452,19 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
         <v>8</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" t="s">
-        <v>14</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1"/>
     <hyperlink ref="C3" r:id="rId2"/>
-    <hyperlink ref="C4" r:id="rId3"/>
-    <hyperlink ref="C5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Validated report update 2025-11-04 15:00
</commit_message>
<xml_diff>
--- a/flagged_segments.xlsx
+++ b/flagged_segments.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="32">
   <si>
     <t>Session</t>
   </si>
@@ -28,19 +28,85 @@
     <t>Category</t>
   </si>
   <si>
+    <t>GMT20251026-075624</t>
+  </si>
+  <si>
     <t>GMT20250821-130122</t>
   </si>
   <si>
+    <t>Hello?</t>
+  </si>
+  <si>
+    <t>Yeah, I'm here, but I cannot see you.</t>
+  </si>
+  <si>
+    <t>I'm not able to… My camera doesn't seem to be working.</t>
+  </si>
+  <si>
+    <t>You can try restarting my computer.</t>
+  </si>
+  <si>
+    <t>Woohoo!</t>
+  </si>
+  <si>
+    <t>It's working now.</t>
+  </si>
+  <si>
+    <t>Hi, can you hear me?</t>
+  </si>
+  <si>
+    <t>… can't… oh, can you hear me?</t>
+  </si>
+  <si>
+    <t>Nope.</t>
+  </si>
+  <si>
+    <t>Hello, can you hear me? I can hear you.</t>
+  </si>
+  <si>
+    <t>Can you hear me?</t>
+  </si>
+  <si>
+    <t>Oh, interesting. I'll double-check my audio, but I think… oh, you can't hear me, one second.</t>
+  </si>
+  <si>
+    <t>Gotcha. I think my Wi-Fi should be fine.</t>
+  </si>
+  <si>
+    <t>Oh, alright, awesome. Okay, before we get started, any questions on equilibrium reactions? We went over them quite extensively last time, and we did a couple examples, but then we also sort of talked about altering conditions.</t>
+  </si>
+  <si>
+    <t>There's, like, slight cuts of….</t>
+  </si>
+  <si>
     <t>Oh my god, I'm so sorry, I don't know why. Some meeting rooms… in some meeting rooms in my department, the connection is weird. If I start lagging at any point, let me know again. But yeah, we lost, like.</t>
   </si>
   <si>
-    <t>ask them not to charge you for this class, and then I can give you a full makeup class, instead of this one, because it's unfair to just have you not understand half the things I'm saying.</t>
+    <t>Yeah, I think it's delayed.</t>
+  </si>
+  <si>
+    <t>Does that make sense?</t>
+  </si>
+  <si>
+    <t>Alright. So basically, with reversible reactions, the reason why your product can go back to being reactants is because of this differential energy state between them.</t>
+  </si>
+  <si>
+    <t>Yes, yes, yeah, I'm just apologizing again, and please also apologize to your parents for me, but we'll make sure to sort this out with the team, and we'll do a makeup class for sure.</t>
+  </si>
+  <si>
+    <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20251026-075624_validated_report.html</t>
   </si>
   <si>
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20250821-130122_validated_report.html</t>
   </si>
   <si>
-    <t>Tutor Policy Breach: Payment Outside Platform</t>
+    <t>Technical: Audio Issues</t>
+  </si>
+  <si>
+    <t>Technical: Video Issues</t>
+  </si>
+  <si>
+    <t>Technical: Connectivity Issues</t>
   </si>
   <si>
     <t>View Report</t>
@@ -410,7 +476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -438,13 +504,13 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>8</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -452,19 +518,304 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D12" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" t="s">
-        <v>8</v>
+      <c r="C14" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B15" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D16" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" t="s">
+        <v>5</v>
+      </c>
+      <c r="B17" t="s">
+        <v>20</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D17" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" t="s">
+        <v>5</v>
+      </c>
+      <c r="B18" t="s">
+        <v>21</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D18" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" t="s">
+        <v>5</v>
+      </c>
+      <c r="B19" t="s">
+        <v>22</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D19" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" t="s">
+        <v>5</v>
+      </c>
+      <c r="B20" t="s">
+        <v>23</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D20" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" t="s">
+        <v>5</v>
+      </c>
+      <c r="B21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D21" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" t="s">
+        <v>5</v>
+      </c>
+      <c r="B22" t="s">
+        <v>25</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D22" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1"/>
     <hyperlink ref="C3" r:id="rId2"/>
+    <hyperlink ref="C4" r:id="rId3"/>
+    <hyperlink ref="C5" r:id="rId4"/>
+    <hyperlink ref="C6" r:id="rId5"/>
+    <hyperlink ref="C7" r:id="rId6"/>
+    <hyperlink ref="C8" r:id="rId7"/>
+    <hyperlink ref="C9" r:id="rId8"/>
+    <hyperlink ref="C10" r:id="rId9"/>
+    <hyperlink ref="C11" r:id="rId10"/>
+    <hyperlink ref="C12" r:id="rId11"/>
+    <hyperlink ref="C13" r:id="rId12"/>
+    <hyperlink ref="C14" r:id="rId13"/>
+    <hyperlink ref="C15" r:id="rId14"/>
+    <hyperlink ref="C16" r:id="rId15"/>
+    <hyperlink ref="C17" r:id="rId16"/>
+    <hyperlink ref="C18" r:id="rId17"/>
+    <hyperlink ref="C19" r:id="rId18"/>
+    <hyperlink ref="C20" r:id="rId19"/>
+    <hyperlink ref="C21" r:id="rId20"/>
+    <hyperlink ref="C22" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Validated report update 2025-11-05 21:07
</commit_message>
<xml_diff>
--- a/flagged_segments.xlsx
+++ b/flagged_segments.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="61">
   <si>
     <t>Session</t>
   </si>
@@ -40,16 +40,40 @@
     <t>Yeah, I'm here, but I cannot see you.</t>
   </si>
   <si>
-    <t>I'm not able to… My camera doesn't seem to be working.</t>
-  </si>
-  <si>
-    <t>You can try restarting my computer.</t>
+    <t>I'm not able to get it to work now.</t>
   </si>
   <si>
     <t>Woohoo!</t>
   </si>
   <si>
-    <t>It's working now.</t>
+    <t>Yeah. And something as basic as turning it off and turning it on again can find solutions.</t>
+  </si>
+  <si>
+    <t>Yes, it can often fix it.</t>
+  </si>
+  <si>
+    <t>Then it works.</t>
+  </si>
+  <si>
+    <t>So you don't have a lot of context.</t>
+  </si>
+  <si>
+    <t>So, I… I read a lot of stuff. I read a lot of outside sources.</t>
+  </si>
+  <si>
+    <t>I didn't start reading Unit 4 yet, I was still just reviewing Unit 3. We're starting Unit 4, like, on Monday.</t>
+  </si>
+  <si>
+    <t>the Ottoman Empire was a political and religious and economic force. And what do you think ended the Ottoman Empire?</t>
+  </si>
+  <si>
+    <t>Bit of it, because they took, like, engineers and stuff to make stuff.</t>
+  </si>
+  <si>
+    <t>Yes?</t>
+  </si>
+  <si>
+    <t>But they just borrowed the technology that had been used before them.</t>
   </si>
   <si>
     <t>Hi, can you hear me?</t>
@@ -64,34 +88,73 @@
     <t>Hello, can you hear me? I can hear you.</t>
   </si>
   <si>
+    <t>I can hear you.</t>
+  </si>
+  <si>
     <t>Can you hear me?</t>
   </si>
   <si>
     <t>Oh, interesting. I'll double-check my audio, but I think… oh, you can't hear me, one second.</t>
   </si>
   <si>
+    <t>Hello? I don't know if you can hear me, but I'll leave the call and just join back.</t>
+  </si>
+  <si>
+    <t>Yes, can you hear me?</t>
+  </si>
+  <si>
+    <t>Oh, alright, awesome. Yes, I can hear you, can you hear me?</t>
+  </si>
+  <si>
+    <t>Yeah, I can hear you, Vuz, it's just really delayed.</t>
+  </si>
+  <si>
     <t>Gotcha. I think my Wi-Fi should be fine.</t>
   </si>
   <si>
-    <t>Oh, alright, awesome. Okay, before we get started, any questions on equilibrium reactions? We went over them quite extensively last time, and we did a couple examples, but then we also sort of talked about altering conditions.</t>
+    <t>Oh, I see, I see, okay. Good. But is it lagging? Is the Wi-Fi fine now?</t>
+  </si>
+  <si>
+    <t>Because the reversible reactions can go back, and in normal reactions, the products can't, react back to the original, reactants.</t>
   </si>
   <si>
     <t>There's, like, slight cuts of….</t>
   </si>
   <si>
+    <t>I am definitely lagging. Or, or I don't know, there's something off.</t>
+  </si>
+  <si>
+    <t>Wi-Fi or yours. Give me just a second, I'll try to restart my Wi-Fi very quickly.</t>
+  </si>
+  <si>
+    <t>Yeah, can you hear me better now?</t>
+  </si>
+  <si>
+    <t>find another meeting room. I don't know.</t>
+  </si>
+  <si>
     <t>Oh my god, I'm so sorry, I don't know why. Some meeting rooms… in some meeting rooms in my department, the connection is weird. If I start lagging at any point, let me know again. But yeah, we lost, like.</t>
   </si>
   <si>
-    <t>Yeah, I think it's delayed.</t>
-  </si>
-  <si>
-    <t>Does that make sense?</t>
-  </si>
-  <si>
-    <t>Alright. So basically, with reversible reactions, the reason why your product can go back to being reactants is because of this differential energy state between them.</t>
-  </si>
-  <si>
-    <t>Yes, yes, yeah, I'm just apologizing again, and please also apologize to your parents for me, but we'll make sure to sort this out with the team, and we'll do a makeup class for sure.</t>
+    <t>5 to 10 minutes. I will have to leave by, like, 3 sharp, so I'm really sorry about that. But we can definitely stay on longer next week, because I don't have a meeting right after our session, because usually we meet at 4. Does that work?</t>
+  </si>
+  <si>
+    <t>It's unfair to you if we just go on like this for the next 30, 40 minutes of this session. If the internet issue continues happening, then I'll just ask them to, like, not charge you for the session. Hello? Can you hear me?</t>
+  </si>
+  <si>
+    <t>ask them not to charge you for this class, and then I can give you a full makeup class, instead of this one, because it's unfair to just have you not understand half the things I'm saying.</t>
+  </si>
+  <si>
+    <t>I think it's not from this end, because my wife and I are showing that everything.</t>
+  </si>
+  <si>
+    <t>Okay?</t>
+  </si>
+  <si>
+    <t>I think… okay. I think the minute I start actually explaining things, you start, like, you start getting frozen in my screen, but I'm just gonna keep saying things, and if at some point you can't understand what I'm saying, just stop me.</t>
+  </si>
+  <si>
+    <t>How do we define stability in chemistry?</t>
   </si>
   <si>
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20251026-075624_validated_report.html</t>
@@ -107,6 +170,30 @@
   </si>
   <si>
     <t>Technical: Connectivity Issues</t>
+  </si>
+  <si>
+    <t>Session Quality: Tutor Monologue</t>
+  </si>
+  <si>
+    <t>Student Behavior Issues: Homework Non-Completion</t>
+  </si>
+  <si>
+    <t>Safety: Illegal Activities</t>
+  </si>
+  <si>
+    <t>Other: Parent Over-Involvement</t>
+  </si>
+  <si>
+    <t>Administrative: Session Cancellation / Rescheduling</t>
+  </si>
+  <si>
+    <t>Administrative: Payment Adjustments</t>
+  </si>
+  <si>
+    <t>Session Quality: Off-Topic Discussion</t>
+  </si>
+  <si>
+    <t>Technical: Session Quality</t>
   </si>
   <si>
     <t>View Report</t>
@@ -476,7 +563,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D47"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -507,10 +594,10 @@
         <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="D2" t="s">
-        <v>28</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -521,10 +608,10 @@
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="D3" t="s">
-        <v>29</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -535,10 +622,10 @@
         <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="D4" t="s">
-        <v>29</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -546,13 +633,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="D5" t="s">
-        <v>29</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -560,13 +647,13 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="D6" t="s">
-        <v>30</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -574,153 +661,153 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="D7" t="s">
-        <v>30</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="D8" t="s">
-        <v>28</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="D9" t="s">
-        <v>28</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="D10" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="D11" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B12" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="D12" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="D13" t="s">
-        <v>28</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B14" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="D14" t="s">
-        <v>28</v>
+        <v>54</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="D15" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="D16" t="s">
-        <v>28</v>
+        <v>55</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="D17" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -728,13 +815,13 @@
         <v>5</v>
       </c>
       <c r="B18" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="D18" t="s">
-        <v>30</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -742,13 +829,13 @@
         <v>5</v>
       </c>
       <c r="B19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="D19" t="s">
-        <v>30</v>
+        <v>49</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -756,13 +843,13 @@
         <v>5</v>
       </c>
       <c r="B20" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="D20" t="s">
-        <v>30</v>
+        <v>49</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -770,13 +857,13 @@
         <v>5</v>
       </c>
       <c r="B21" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="D21" t="s">
-        <v>30</v>
+        <v>49</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -784,13 +871,363 @@
         <v>5</v>
       </c>
       <c r="B22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D22" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" t="s">
+        <v>5</v>
+      </c>
+      <c r="B23" t="s">
+        <v>24</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D23" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B24" t="s">
         <v>25</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C24" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D24" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" t="s">
+        <v>5</v>
+      </c>
+      <c r="B25" t="s">
+        <v>26</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D25" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" t="s">
+        <v>5</v>
+      </c>
+      <c r="B26" t="s">
+        <v>6</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D26" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" t="s">
+        <v>5</v>
+      </c>
+      <c r="B27" t="s">
+        <v>27</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D27" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" t="s">
+        <v>5</v>
+      </c>
+      <c r="B28" t="s">
+        <v>6</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D28" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" t="s">
+        <v>5</v>
+      </c>
+      <c r="B29" t="s">
+        <v>28</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D29" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="A30" t="s">
+        <v>5</v>
+      </c>
+      <c r="B30" t="s">
+        <v>29</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D30" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31" t="s">
+        <v>5</v>
+      </c>
+      <c r="B31" t="s">
+        <v>30</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D31" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
+      <c r="A32" t="s">
+        <v>5</v>
+      </c>
+      <c r="B32" t="s">
         <v>31</v>
       </c>
-      <c r="D22" t="s">
-        <v>30</v>
+      <c r="C32" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D32" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" t="s">
+        <v>5</v>
+      </c>
+      <c r="B33" t="s">
+        <v>32</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D33" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4">
+      <c r="A34" t="s">
+        <v>5</v>
+      </c>
+      <c r="B34" t="s">
+        <v>33</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D34" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4">
+      <c r="A35" t="s">
+        <v>5</v>
+      </c>
+      <c r="B35" t="s">
+        <v>34</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D35" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4">
+      <c r="A36" t="s">
+        <v>5</v>
+      </c>
+      <c r="B36" t="s">
+        <v>35</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D36" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
+      <c r="A37" t="s">
+        <v>5</v>
+      </c>
+      <c r="B37" t="s">
+        <v>36</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D37" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
+      <c r="A38" t="s">
+        <v>5</v>
+      </c>
+      <c r="B38" t="s">
+        <v>37</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D38" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
+      <c r="A39" t="s">
+        <v>5</v>
+      </c>
+      <c r="B39" t="s">
+        <v>38</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D39" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
+      <c r="A40" t="s">
+        <v>5</v>
+      </c>
+      <c r="B40" t="s">
+        <v>39</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D40" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
+      <c r="A41" t="s">
+        <v>5</v>
+      </c>
+      <c r="B41" t="s">
+        <v>40</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D41" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
+      <c r="A42" t="s">
+        <v>5</v>
+      </c>
+      <c r="B42" t="s">
+        <v>41</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D42" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
+      <c r="A43" t="s">
+        <v>5</v>
+      </c>
+      <c r="B43" t="s">
+        <v>42</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D43" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4">
+      <c r="A44" t="s">
+        <v>5</v>
+      </c>
+      <c r="B44" t="s">
+        <v>43</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D44" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4">
+      <c r="A45" t="s">
+        <v>5</v>
+      </c>
+      <c r="B45" t="s">
+        <v>44</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D45" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4">
+      <c r="A46" t="s">
+        <v>5</v>
+      </c>
+      <c r="B46" t="s">
+        <v>45</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D46" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4">
+      <c r="A47" t="s">
+        <v>5</v>
+      </c>
+      <c r="B47" t="s">
+        <v>46</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D47" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -816,6 +1253,31 @@
     <hyperlink ref="C20" r:id="rId19"/>
     <hyperlink ref="C21" r:id="rId20"/>
     <hyperlink ref="C22" r:id="rId21"/>
+    <hyperlink ref="C23" r:id="rId22"/>
+    <hyperlink ref="C24" r:id="rId23"/>
+    <hyperlink ref="C25" r:id="rId24"/>
+    <hyperlink ref="C26" r:id="rId25"/>
+    <hyperlink ref="C27" r:id="rId26"/>
+    <hyperlink ref="C28" r:id="rId27"/>
+    <hyperlink ref="C29" r:id="rId28"/>
+    <hyperlink ref="C30" r:id="rId29"/>
+    <hyperlink ref="C31" r:id="rId30"/>
+    <hyperlink ref="C32" r:id="rId31"/>
+    <hyperlink ref="C33" r:id="rId32"/>
+    <hyperlink ref="C34" r:id="rId33"/>
+    <hyperlink ref="C35" r:id="rId34"/>
+    <hyperlink ref="C36" r:id="rId35"/>
+    <hyperlink ref="C37" r:id="rId36"/>
+    <hyperlink ref="C38" r:id="rId37"/>
+    <hyperlink ref="C39" r:id="rId38"/>
+    <hyperlink ref="C40" r:id="rId39"/>
+    <hyperlink ref="C41" r:id="rId40"/>
+    <hyperlink ref="C42" r:id="rId41"/>
+    <hyperlink ref="C43" r:id="rId42"/>
+    <hyperlink ref="C44" r:id="rId43"/>
+    <hyperlink ref="C45" r:id="rId44"/>
+    <hyperlink ref="C46" r:id="rId45"/>
+    <hyperlink ref="C47" r:id="rId46"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Validated report update 2025-11-05 21:52
</commit_message>
<xml_diff>
--- a/flagged_segments.xlsx
+++ b/flagged_segments.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="42">
   <si>
     <t>Session</t>
   </si>
@@ -40,40 +40,16 @@
     <t>Yeah, I'm here, but I cannot see you.</t>
   </si>
   <si>
+    <t>I'm not able to… My camera doesn't seem to be working.</t>
+  </si>
+  <si>
     <t>I'm not able to get it to work now.</t>
   </si>
   <si>
-    <t>Woohoo!</t>
-  </si>
-  <si>
-    <t>Yeah. And something as basic as turning it off and turning it on again can find solutions.</t>
-  </si>
-  <si>
-    <t>Yes, it can often fix it.</t>
-  </si>
-  <si>
-    <t>Then it works.</t>
-  </si>
-  <si>
-    <t>So you don't have a lot of context.</t>
-  </si>
-  <si>
-    <t>So, I… I read a lot of stuff. I read a lot of outside sources.</t>
-  </si>
-  <si>
-    <t>I didn't start reading Unit 4 yet, I was still just reviewing Unit 3. We're starting Unit 4, like, on Monday.</t>
-  </si>
-  <si>
-    <t>the Ottoman Empire was a political and religious and economic force. And what do you think ended the Ottoman Empire?</t>
-  </si>
-  <si>
-    <t>Bit of it, because they took, like, engineers and stuff to make stuff.</t>
-  </si>
-  <si>
-    <t>Yes?</t>
-  </si>
-  <si>
-    <t>But they just borrowed the technology that had been used before them.</t>
+    <t>I'm trying to turn on my kit.</t>
+  </si>
+  <si>
+    <t>One…</t>
   </si>
   <si>
     <t>Hi, can you hear me?</t>
@@ -88,24 +64,21 @@
     <t>Hello, can you hear me? I can hear you.</t>
   </si>
   <si>
-    <t>I can hear you.</t>
+    <t>Yes, can you hear me?</t>
   </si>
   <si>
     <t>Can you hear me?</t>
   </si>
   <si>
+    <t>I can, yeah, but can you hear me?</t>
+  </si>
+  <si>
     <t>Oh, interesting. I'll double-check my audio, but I think… oh, you can't hear me, one second.</t>
   </si>
   <si>
     <t>Hello? I don't know if you can hear me, but I'll leave the call and just join back.</t>
   </si>
   <si>
-    <t>Yes, can you hear me?</t>
-  </si>
-  <si>
-    <t>Oh, alright, awesome. Yes, I can hear you, can you hear me?</t>
-  </si>
-  <si>
     <t>Yeah, I can hear you, Vuz, it's just really delayed.</t>
   </si>
   <si>
@@ -115,46 +88,34 @@
     <t>Oh, I see, I see, okay. Good. But is it lagging? Is the Wi-Fi fine now?</t>
   </si>
   <si>
-    <t>Because the reversible reactions can go back, and in normal reactions, the products can't, react back to the original, reactants.</t>
+    <t>Just so you have a bit more of a head start, and that way we'd be ahead of the material… we're gonna be ahead of the material in class anyway, since you started in summer, but we could be more ahead.</t>
+  </si>
+  <si>
+    <t>Can you hear me properly? I can't tell if I'm lagging or not.</t>
   </si>
   <si>
     <t>There's, like, slight cuts of….</t>
   </si>
   <si>
-    <t>I am definitely lagging. Or, or I don't know, there's something off.</t>
-  </si>
-  <si>
-    <t>Wi-Fi or yours. Give me just a second, I'll try to restart my Wi-Fi very quickly.</t>
-  </si>
-  <si>
-    <t>Yeah, can you hear me better now?</t>
-  </si>
-  <si>
-    <t>find another meeting room. I don't know.</t>
-  </si>
-  <si>
-    <t>Oh my god, I'm so sorry, I don't know why. Some meeting rooms… in some meeting rooms in my department, the connection is weird. If I start lagging at any point, let me know again. But yeah, we lost, like.</t>
-  </si>
-  <si>
-    <t>5 to 10 minutes. I will have to leave by, like, 3 sharp, so I'm really sorry about that. But we can definitely stay on longer next week, because I don't have a meeting right after our session, because usually we meet at 4. Does that work?</t>
-  </si>
-  <si>
-    <t>It's unfair to you if we just go on like this for the next 30, 40 minutes of this session. If the internet issue continues happening, then I'll just ask them to, like, not charge you for the session. Hello? Can you hear me?</t>
-  </si>
-  <si>
-    <t>ask them not to charge you for this class, and then I can give you a full makeup class, instead of this one, because it's unfair to just have you not understand half the things I'm saying.</t>
-  </si>
-  <si>
-    <t>I think it's not from this end, because my wife and I are showing that everything.</t>
-  </si>
-  <si>
-    <t>Okay?</t>
-  </si>
-  <si>
-    <t>I think… okay. I think the minute I start actually explaining things, you start, like, you start getting frozen in my screen, but I'm just gonna keep saying things, and if at some point you can't understand what I'm saying, just stop me.</t>
-  </si>
-  <si>
-    <t>How do we define stability in chemistry?</t>
+    <t>I can't tell if the issue is… I can't tell if it's… the issue is my…</t>
+  </si>
+  <si>
+    <t>Hello? Now I can hear you, yeah. I was trying to find out what happened.</t>
+  </si>
+  <si>
+    <t>Let me try and sort this out.</t>
+  </si>
+  <si>
+    <t>I think…</t>
+  </si>
+  <si>
+    <t>So, would you… I think it's unfair to you… let's try to go on for 5 minutes. Can you hear me… can you hear what I'm saying?</t>
+  </si>
+  <si>
+    <t>Is that fine? I think it's just unfair to you that I just talk and you spend, like, half the time deciphering what I'm saying because of internet issues.</t>
+  </si>
+  <si>
+    <t>having, you know, like, the next 30 minutes, and also not being 100% sure, you'll hear what I'm saying in the next 30 minutes.</t>
   </si>
   <si>
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20251026-075624_validated_report.html</t>
@@ -172,28 +133,10 @@
     <t>Technical: Connectivity Issues</t>
   </si>
   <si>
-    <t>Session Quality: Tutor Monologue</t>
-  </si>
-  <si>
-    <t>Student Behavior Issues: Homework Non-Completion</t>
-  </si>
-  <si>
-    <t>Safety: Illegal Activities</t>
-  </si>
-  <si>
-    <t>Other: Parent Over-Involvement</t>
+    <t>Administrative: Payment Adjustments</t>
   </si>
   <si>
     <t>Administrative: Session Cancellation / Rescheduling</t>
-  </si>
-  <si>
-    <t>Administrative: Payment Adjustments</t>
-  </si>
-  <si>
-    <t>Session Quality: Off-Topic Discussion</t>
-  </si>
-  <si>
-    <t>Technical: Session Quality</t>
   </si>
   <si>
     <t>View Report</t>
@@ -563,7 +506,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D47"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -594,10 +537,10 @@
         <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D2" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -608,10 +551,10 @@
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D3" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -622,10 +565,10 @@
         <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D4" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -633,13 +576,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D5" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -650,10 +593,10 @@
         <v>9</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D6" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -661,13 +604,13 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D7" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -675,13 +618,13 @@
         <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D8" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -689,13 +632,13 @@
         <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D9" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -703,13 +646,13 @@
         <v>4</v>
       </c>
       <c r="B10" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D10" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -717,13 +660,13 @@
         <v>4</v>
       </c>
       <c r="B11" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D11" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -731,83 +674,83 @@
         <v>4</v>
       </c>
       <c r="B12" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D12" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B13" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D13" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B14" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D14" t="s">
-        <v>54</v>
+        <v>36</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B15" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D15" t="s">
-        <v>54</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B16" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D16" t="s">
-        <v>55</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B17" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D17" t="s">
-        <v>54</v>
+        <v>36</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -815,13 +758,13 @@
         <v>5</v>
       </c>
       <c r="B18" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D18" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -829,13 +772,13 @@
         <v>5</v>
       </c>
       <c r="B19" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D19" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -843,13 +786,13 @@
         <v>5</v>
       </c>
       <c r="B20" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D20" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -857,13 +800,13 @@
         <v>5</v>
       </c>
       <c r="B21" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D21" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -874,10 +817,10 @@
         <v>6</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D22" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -885,13 +828,13 @@
         <v>5</v>
       </c>
       <c r="B23" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D23" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -899,13 +842,13 @@
         <v>5</v>
       </c>
       <c r="B24" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D24" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -913,13 +856,13 @@
         <v>5</v>
       </c>
       <c r="B25" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D25" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -927,13 +870,13 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D26" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -941,13 +884,13 @@
         <v>5</v>
       </c>
       <c r="B27" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D27" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -955,13 +898,13 @@
         <v>5</v>
       </c>
       <c r="B28" t="s">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D28" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -969,13 +912,13 @@
         <v>5</v>
       </c>
       <c r="B29" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D29" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -983,13 +926,13 @@
         <v>5</v>
       </c>
       <c r="B30" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D30" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -997,13 +940,13 @@
         <v>5</v>
       </c>
       <c r="B31" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D31" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -1011,13 +954,13 @@
         <v>5</v>
       </c>
       <c r="B32" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D32" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -1025,13 +968,13 @@
         <v>5</v>
       </c>
       <c r="B33" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D33" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -1039,13 +982,13 @@
         <v>5</v>
       </c>
       <c r="B34" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D34" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -1053,13 +996,13 @@
         <v>5</v>
       </c>
       <c r="B35" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D35" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -1067,13 +1010,13 @@
         <v>5</v>
       </c>
       <c r="B36" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D36" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -1081,13 +1024,13 @@
         <v>5</v>
       </c>
       <c r="B37" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D37" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -1095,139 +1038,13 @@
         <v>5</v>
       </c>
       <c r="B38" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D38" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4">
-      <c r="A39" t="s">
-        <v>5</v>
-      </c>
-      <c r="B39" t="s">
-        <v>38</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D39" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4">
-      <c r="A40" t="s">
-        <v>5</v>
-      </c>
-      <c r="B40" t="s">
-        <v>39</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D40" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4">
-      <c r="A41" t="s">
-        <v>5</v>
-      </c>
-      <c r="B41" t="s">
         <v>40</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D41" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4">
-      <c r="A42" t="s">
-        <v>5</v>
-      </c>
-      <c r="B42" t="s">
-        <v>41</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D42" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4">
-      <c r="A43" t="s">
-        <v>5</v>
-      </c>
-      <c r="B43" t="s">
-        <v>42</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D43" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4">
-      <c r="A44" t="s">
-        <v>5</v>
-      </c>
-      <c r="B44" t="s">
-        <v>43</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D44" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4">
-      <c r="A45" t="s">
-        <v>5</v>
-      </c>
-      <c r="B45" t="s">
-        <v>44</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D45" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4">
-      <c r="A46" t="s">
-        <v>5</v>
-      </c>
-      <c r="B46" t="s">
-        <v>45</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D46" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4">
-      <c r="A47" t="s">
-        <v>5</v>
-      </c>
-      <c r="B47" t="s">
-        <v>46</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D47" t="s">
-        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1269,15 +1086,6 @@
     <hyperlink ref="C36" r:id="rId35"/>
     <hyperlink ref="C37" r:id="rId36"/>
     <hyperlink ref="C38" r:id="rId37"/>
-    <hyperlink ref="C39" r:id="rId38"/>
-    <hyperlink ref="C40" r:id="rId39"/>
-    <hyperlink ref="C41" r:id="rId40"/>
-    <hyperlink ref="C42" r:id="rId41"/>
-    <hyperlink ref="C43" r:id="rId42"/>
-    <hyperlink ref="C44" r:id="rId43"/>
-    <hyperlink ref="C45" r:id="rId44"/>
-    <hyperlink ref="C46" r:id="rId45"/>
-    <hyperlink ref="C47" r:id="rId46"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Validated report update 2025-11-08 13:19
</commit_message>
<xml_diff>
--- a/flagged_segments.xlsx
+++ b/flagged_segments.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="27">
   <si>
     <t>Session</t>
   </si>
@@ -34,88 +34,46 @@
     <t>GMT20250821-130122</t>
   </si>
   <si>
+    <t>Yeah, I'm here, but I cannot see you.</t>
+  </si>
+  <si>
+    <t>I'm trying to turn on my kit.</t>
+  </si>
+  <si>
+    <t>I'm not able to get it to work now.</t>
+  </si>
+  <si>
+    <t>I'm not able to… My camera doesn't seem to be working.</t>
+  </si>
+  <si>
+    <t>Hi, can you hear me?</t>
+  </si>
+  <si>
+    <t>… can't… oh, can you hear me?</t>
+  </si>
+  <si>
+    <t>Nope.</t>
+  </si>
+  <si>
+    <t>Hello, can you hear me? I can hear you.</t>
+  </si>
+  <si>
     <t>Hello?</t>
   </si>
   <si>
-    <t>Yeah, I'm here, but I cannot see you.</t>
-  </si>
-  <si>
-    <t>I'm not able to… My camera doesn't seem to be working.</t>
-  </si>
-  <si>
-    <t>I'm not able to get it to work now.</t>
-  </si>
-  <si>
-    <t>I'm trying to turn on my kit.</t>
-  </si>
-  <si>
-    <t>One…</t>
-  </si>
-  <si>
-    <t>Hi, can you hear me?</t>
-  </si>
-  <si>
-    <t>… can't… oh, can you hear me?</t>
-  </si>
-  <si>
-    <t>Nope.</t>
-  </si>
-  <si>
-    <t>Hello, can you hear me? I can hear you.</t>
-  </si>
-  <si>
     <t>Yes, can you hear me?</t>
   </si>
   <si>
-    <t>Can you hear me?</t>
-  </si>
-  <si>
-    <t>I can, yeah, but can you hear me?</t>
-  </si>
-  <si>
-    <t>Oh, interesting. I'll double-check my audio, but I think… oh, you can't hear me, one second.</t>
-  </si>
-  <si>
     <t>Hello? I don't know if you can hear me, but I'll leave the call and just join back.</t>
   </si>
   <si>
     <t>Yeah, I can hear you, Vuz, it's just really delayed.</t>
   </si>
   <si>
-    <t>Gotcha. I think my Wi-Fi should be fine.</t>
-  </si>
-  <si>
-    <t>Oh, I see, I see, okay. Good. But is it lagging? Is the Wi-Fi fine now?</t>
-  </si>
-  <si>
-    <t>Just so you have a bit more of a head start, and that way we'd be ahead of the material… we're gonna be ahead of the material in class anyway, since you started in summer, but we could be more ahead.</t>
-  </si>
-  <si>
-    <t>Can you hear me properly? I can't tell if I'm lagging or not.</t>
-  </si>
-  <si>
-    <t>There's, like, slight cuts of….</t>
-  </si>
-  <si>
-    <t>I can't tell if the issue is… I can't tell if it's… the issue is my…</t>
-  </si>
-  <si>
-    <t>Hello? Now I can hear you, yeah. I was trying to find out what happened.</t>
-  </si>
-  <si>
-    <t>Let me try and sort this out.</t>
-  </si>
-  <si>
-    <t>I think…</t>
-  </si>
-  <si>
-    <t>So, would you… I think it's unfair to you… let's try to go on for 5 minutes. Can you hear me… can you hear what I'm saying?</t>
-  </si>
-  <si>
-    <t>Is that fine? I think it's just unfair to you that I just talk and you spend, like, half the time deciphering what I'm saying because of internet issues.</t>
-  </si>
-  <si>
-    <t>having, you know, like, the next 30 minutes, and also not being 100% sure, you'll hear what I'm saying in the next 30 minutes.</t>
+    <t>Wi-Fi or yours. Give me just a second, I'll try to restart my Wi-Fi very quickly.</t>
+  </si>
+  <si>
+    <t>It's unfair to you if we just go on like this for the next 30, 40 minutes of this session. If the internet issue continues happening, then I'll just ask them to, like, not charge you for the session. Hello? Can you hear me?</t>
   </si>
   <si>
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20251026-075624_validated_report.html</t>
@@ -124,19 +82,16 @@
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20250821-130122_validated_report.html</t>
   </si>
   <si>
+    <t>Technical: Video Issues</t>
+  </si>
+  <si>
     <t>Technical: Audio Issues</t>
   </si>
   <si>
-    <t>Technical: Video Issues</t>
-  </si>
-  <si>
     <t>Technical: Connectivity Issues</t>
   </si>
   <si>
     <t>Administrative: Payment Adjustments</t>
-  </si>
-  <si>
-    <t>Administrative: Session Cancellation / Rescheduling</t>
   </si>
   <si>
     <t>View Report</t>
@@ -506,7 +461,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -537,10 +492,10 @@
         <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D2" t="s">
-        <v>36</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -551,10 +506,10 @@
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D3" t="s">
-        <v>37</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -565,10 +520,10 @@
         <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D4" t="s">
-        <v>37</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -576,111 +531,111 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D5" t="s">
-        <v>37</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D6" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D7" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D8" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B9" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D9" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B10" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D10" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B11" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D11" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B12" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D12" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -688,13 +643,13 @@
         <v>5</v>
       </c>
       <c r="B13" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D13" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -702,13 +657,13 @@
         <v>5</v>
       </c>
       <c r="B14" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D14" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -716,335 +671,13 @@
         <v>5</v>
       </c>
       <c r="B15" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D15" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" t="s">
-        <v>5</v>
-      </c>
-      <c r="B16" t="s">
-        <v>15</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D16" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="A17" t="s">
-        <v>5</v>
-      </c>
-      <c r="B17" t="s">
-        <v>6</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D17" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4">
-      <c r="A18" t="s">
-        <v>5</v>
-      </c>
-      <c r="B18" t="s">
-        <v>16</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D18" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4">
-      <c r="A19" t="s">
-        <v>5</v>
-      </c>
-      <c r="B19" t="s">
-        <v>17</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D19" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4">
-      <c r="A20" t="s">
-        <v>5</v>
-      </c>
-      <c r="B20" t="s">
-        <v>18</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D20" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4">
-      <c r="A21" t="s">
-        <v>5</v>
-      </c>
-      <c r="B21" t="s">
-        <v>19</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D21" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4">
-      <c r="A22" t="s">
-        <v>5</v>
-      </c>
-      <c r="B22" t="s">
-        <v>6</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D22" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4">
-      <c r="A23" t="s">
-        <v>5</v>
-      </c>
-      <c r="B23" t="s">
-        <v>20</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D23" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4">
-      <c r="A24" t="s">
-        <v>5</v>
-      </c>
-      <c r="B24" t="s">
-        <v>6</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D24" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4">
-      <c r="A25" t="s">
-        <v>5</v>
-      </c>
-      <c r="B25" t="s">
-        <v>16</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D25" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4">
-      <c r="A26" t="s">
-        <v>5</v>
-      </c>
-      <c r="B26" t="s">
-        <v>21</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D26" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4">
-      <c r="A27" t="s">
-        <v>5</v>
-      </c>
-      <c r="B27" t="s">
-        <v>22</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D27" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4">
-      <c r="A28" t="s">
-        <v>5</v>
-      </c>
-      <c r="B28" t="s">
-        <v>23</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D28" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4">
-      <c r="A29" t="s">
-        <v>5</v>
-      </c>
-      <c r="B29" t="s">
-        <v>24</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D29" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4">
-      <c r="A30" t="s">
-        <v>5</v>
-      </c>
-      <c r="B30" t="s">
         <v>25</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D30" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4">
-      <c r="A31" t="s">
-        <v>5</v>
-      </c>
-      <c r="B31" t="s">
-        <v>26</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D31" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4">
-      <c r="A32" t="s">
-        <v>5</v>
-      </c>
-      <c r="B32" t="s">
-        <v>27</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D32" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4">
-      <c r="A33" t="s">
-        <v>5</v>
-      </c>
-      <c r="B33" t="s">
-        <v>28</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D33" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4">
-      <c r="A34" t="s">
-        <v>5</v>
-      </c>
-      <c r="B34" t="s">
-        <v>29</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D34" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4">
-      <c r="A35" t="s">
-        <v>5</v>
-      </c>
-      <c r="B35" t="s">
-        <v>30</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D35" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4">
-      <c r="A36" t="s">
-        <v>5</v>
-      </c>
-      <c r="B36" t="s">
-        <v>31</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D36" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4">
-      <c r="A37" t="s">
-        <v>5</v>
-      </c>
-      <c r="B37" t="s">
-        <v>32</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D37" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4">
-      <c r="A38" t="s">
-        <v>5</v>
-      </c>
-      <c r="B38" t="s">
-        <v>33</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D38" t="s">
-        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -1063,29 +696,6 @@
     <hyperlink ref="C13" r:id="rId12"/>
     <hyperlink ref="C14" r:id="rId13"/>
     <hyperlink ref="C15" r:id="rId14"/>
-    <hyperlink ref="C16" r:id="rId15"/>
-    <hyperlink ref="C17" r:id="rId16"/>
-    <hyperlink ref="C18" r:id="rId17"/>
-    <hyperlink ref="C19" r:id="rId18"/>
-    <hyperlink ref="C20" r:id="rId19"/>
-    <hyperlink ref="C21" r:id="rId20"/>
-    <hyperlink ref="C22" r:id="rId21"/>
-    <hyperlink ref="C23" r:id="rId22"/>
-    <hyperlink ref="C24" r:id="rId23"/>
-    <hyperlink ref="C25" r:id="rId24"/>
-    <hyperlink ref="C26" r:id="rId25"/>
-    <hyperlink ref="C27" r:id="rId26"/>
-    <hyperlink ref="C28" r:id="rId27"/>
-    <hyperlink ref="C29" r:id="rId28"/>
-    <hyperlink ref="C30" r:id="rId29"/>
-    <hyperlink ref="C31" r:id="rId30"/>
-    <hyperlink ref="C32" r:id="rId31"/>
-    <hyperlink ref="C33" r:id="rId32"/>
-    <hyperlink ref="C34" r:id="rId33"/>
-    <hyperlink ref="C35" r:id="rId34"/>
-    <hyperlink ref="C36" r:id="rId35"/>
-    <hyperlink ref="C37" r:id="rId36"/>
-    <hyperlink ref="C38" r:id="rId37"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Validated report update 2025-11-08 14:19
</commit_message>
<xml_diff>
--- a/flagged_segments.xlsx
+++ b/flagged_segments.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="21">
   <si>
     <t>Session</t>
   </si>
@@ -37,45 +37,24 @@
     <t>Yeah, I'm here, but I cannot see you.</t>
   </si>
   <si>
-    <t>I'm trying to turn on my kit.</t>
-  </si>
-  <si>
-    <t>I'm not able to get it to work now.</t>
-  </si>
-  <si>
     <t>I'm not able to… My camera doesn't seem to be working.</t>
   </si>
   <si>
+    <t>You can try restarting my computer.</t>
+  </si>
+  <si>
     <t>Hi, can you hear me?</t>
   </si>
   <si>
-    <t>… can't… oh, can you hear me?</t>
-  </si>
-  <si>
-    <t>Nope.</t>
-  </si>
-  <si>
-    <t>Hello, can you hear me? I can hear you.</t>
-  </si>
-  <si>
-    <t>Hello?</t>
-  </si>
-  <si>
-    <t>Yes, can you hear me?</t>
-  </si>
-  <si>
-    <t>Hello? I don't know if you can hear me, but I'll leave the call and just join back.</t>
-  </si>
-  <si>
     <t>Yeah, I can hear you, Vuz, it's just really delayed.</t>
   </si>
   <si>
-    <t>Wi-Fi or yours. Give me just a second, I'll try to restart my Wi-Fi very quickly.</t>
-  </si>
-  <si>
     <t>It's unfair to you if we just go on like this for the next 30, 40 minutes of this session. If the internet issue continues happening, then I'll just ask them to, like, not charge you for the session. Hello? Can you hear me?</t>
   </si>
   <si>
+    <t>So, what I'm saying is, I'll ask the team to cancel the session from our end.</t>
+  </si>
+  <si>
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20251026-075624_validated_report.html</t>
   </si>
   <si>
@@ -85,13 +64,16 @@
     <t>Technical: Video Issues</t>
   </si>
   <si>
+    <t>Technical: Connectivity Issues</t>
+  </si>
+  <si>
     <t>Technical: Audio Issues</t>
   </si>
   <si>
-    <t>Technical: Connectivity Issues</t>
-  </si>
-  <si>
     <t>Administrative: Payment Adjustments</t>
+  </si>
+  <si>
+    <t>Administrative: Session Cancellation / Rescheduling</t>
   </si>
   <si>
     <t>View Report</t>
@@ -461,7 +443,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -492,10 +474,10 @@
         <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D2" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -506,10 +488,10 @@
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D3" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -520,24 +502,24 @@
         <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D4" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -548,10 +530,10 @@
         <v>10</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D6" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -562,10 +544,10 @@
         <v>11</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D7" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -576,108 +558,10 @@
         <v>12</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D8" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D9" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" t="s">
-        <v>5</v>
-      </c>
-      <c r="B10" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D10" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" t="s">
-        <v>5</v>
-      </c>
-      <c r="B11" t="s">
-        <v>15</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D11" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" t="s">
-        <v>5</v>
-      </c>
-      <c r="B12" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D12" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="A13" t="s">
-        <v>5</v>
-      </c>
-      <c r="B13" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D13" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" t="s">
-        <v>5</v>
-      </c>
-      <c r="B14" t="s">
-        <v>18</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D14" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="A15" t="s">
-        <v>5</v>
-      </c>
-      <c r="B15" t="s">
         <v>19</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D15" t="s">
-        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -689,13 +573,6 @@
     <hyperlink ref="C6" r:id="rId5"/>
     <hyperlink ref="C7" r:id="rId6"/>
     <hyperlink ref="C8" r:id="rId7"/>
-    <hyperlink ref="C9" r:id="rId8"/>
-    <hyperlink ref="C10" r:id="rId9"/>
-    <hyperlink ref="C11" r:id="rId10"/>
-    <hyperlink ref="C12" r:id="rId11"/>
-    <hyperlink ref="C13" r:id="rId12"/>
-    <hyperlink ref="C14" r:id="rId13"/>
-    <hyperlink ref="C15" r:id="rId14"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Validated report update 2025-11-08 14:22
</commit_message>
<xml_diff>
--- a/flagged_segments.xlsx
+++ b/flagged_segments.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="26">
   <si>
     <t>Session</t>
   </si>
@@ -34,25 +34,43 @@
     <t>GMT20250821-130122</t>
   </si>
   <si>
+    <t>Ram?</t>
+  </si>
+  <si>
+    <t>Hello.</t>
+  </si>
+  <si>
     <t>Yeah, I'm here, but I cannot see you.</t>
   </si>
   <si>
+    <t>I'm trying to turn on my kit.</t>
+  </si>
+  <si>
+    <t>I'm not able to get it to work now.</t>
+  </si>
+  <si>
     <t>I'm not able to… My camera doesn't seem to be working.</t>
   </si>
   <si>
-    <t>You can try restarting my computer.</t>
+    <t>Yeah. And something as basic as turning it off and turning it on again can find solutions.</t>
   </si>
   <si>
     <t>Hi, can you hear me?</t>
   </si>
   <si>
+    <t>… can't… oh, can you hear me?</t>
+  </si>
+  <si>
+    <t>Hello, can you hear me? I can hear you.</t>
+  </si>
+  <si>
     <t>Yeah, I can hear you, Vuz, it's just really delayed.</t>
   </si>
   <si>
-    <t>It's unfair to you if we just go on like this for the next 30, 40 minutes of this session. If the internet issue continues happening, then I'll just ask them to, like, not charge you for the session. Hello? Can you hear me?</t>
-  </si>
-  <si>
-    <t>So, what I'm saying is, I'll ask the team to cancel the session from our end.</t>
+    <t>There's, like, slight cuts of….</t>
+  </si>
+  <si>
+    <t>Yeah, I can't tell… I can't tell if I'm the one that's lagging, or if it's your… if it's your Wi-Fi, I'm….</t>
   </si>
   <si>
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20251026-075624_validated_report.html</t>
@@ -61,19 +79,16 @@
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20250821-130122_validated_report.html</t>
   </si>
   <si>
+    <t>Technical: Audio Issues</t>
+  </si>
+  <si>
     <t>Technical: Video Issues</t>
   </si>
   <si>
+    <t>Technical: General Issue</t>
+  </si>
+  <si>
     <t>Technical: Connectivity Issues</t>
-  </si>
-  <si>
-    <t>Technical: Audio Issues</t>
-  </si>
-  <si>
-    <t>Administrative: Payment Adjustments</t>
-  </si>
-  <si>
-    <t>Administrative: Session Cancellation / Rescheduling</t>
   </si>
   <si>
     <t>View Report</t>
@@ -443,7 +458,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -474,10 +489,10 @@
         <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -488,10 +503,10 @@
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="D3" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -502,66 +517,150 @@
         <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="D4" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="D5" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" t="s">
         <v>10</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="D6" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="D7" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B8" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="D8" t="s">
-        <v>19</v>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D13" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -573,6 +672,12 @@
     <hyperlink ref="C6" r:id="rId5"/>
     <hyperlink ref="C7" r:id="rId6"/>
     <hyperlink ref="C8" r:id="rId7"/>
+    <hyperlink ref="C9" r:id="rId8"/>
+    <hyperlink ref="C10" r:id="rId9"/>
+    <hyperlink ref="C11" r:id="rId10"/>
+    <hyperlink ref="C12" r:id="rId11"/>
+    <hyperlink ref="C13" r:id="rId12"/>
+    <hyperlink ref="C14" r:id="rId13"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Validated report update 2025-11-08 19:00
</commit_message>
<xml_diff>
--- a/flagged_segments.xlsx
+++ b/flagged_segments.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="21">
   <si>
     <t>Session</t>
   </si>
@@ -34,43 +34,31 @@
     <t>GMT20250821-130122</t>
   </si>
   <si>
-    <t>Ram?</t>
-  </si>
-  <si>
-    <t>Hello.</t>
-  </si>
-  <si>
     <t>Yeah, I'm here, but I cannot see you.</t>
   </si>
   <si>
     <t>I'm trying to turn on my kit.</t>
   </si>
   <si>
-    <t>I'm not able to get it to work now.</t>
-  </si>
-  <si>
     <t>I'm not able to… My camera doesn't seem to be working.</t>
   </si>
   <si>
-    <t>Yeah. And something as basic as turning it off and turning it on again can find solutions.</t>
-  </si>
-  <si>
-    <t>Hi, can you hear me?</t>
+    <t>You can try restarting my computer.</t>
   </si>
   <si>
     <t>… can't… oh, can you hear me?</t>
   </si>
   <si>
-    <t>Hello, can you hear me? I can hear you.</t>
-  </si>
-  <si>
-    <t>Yeah, I can hear you, Vuz, it's just really delayed.</t>
-  </si>
-  <si>
-    <t>There's, like, slight cuts of….</t>
-  </si>
-  <si>
-    <t>Yeah, I can't tell… I can't tell if I'm the one that's lagging, or if it's your… if it's your Wi-Fi, I'm….</t>
+    <t>Yeah, yeah, no, now it's… now it's better. I think the reason I couldn't hear you before is because before I joined the meeting, I didn't click on my headphones, so I was trying to play through my laptop, and it was me.</t>
+  </si>
+  <si>
+    <t>Is it better now?</t>
+  </si>
+  <si>
+    <t>Yeah, the last couple seconds have been okay.</t>
+  </si>
+  <si>
+    <t>What do you think is this… what do you think does this energy makeup look like for reactions that are actually reversible and not complete reactions like this one?</t>
   </si>
   <si>
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20251026-075624_validated_report.html</t>
@@ -79,13 +67,10 @@
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20250821-130122_validated_report.html</t>
   </si>
   <si>
+    <t>Technical: Video Issues</t>
+  </si>
+  <si>
     <t>Technical: Audio Issues</t>
-  </si>
-  <si>
-    <t>Technical: Video Issues</t>
-  </si>
-  <si>
-    <t>Technical: General Issue</t>
   </si>
   <si>
     <t>Technical: Connectivity Issues</t>
@@ -458,7 +443,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -489,10 +474,10 @@
         <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -503,10 +488,10 @@
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D3" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -517,10 +502,10 @@
         <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D4" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -531,52 +516,52 @@
         <v>9</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B6" t="s">
         <v>10</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D6" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B7" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D7" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B8" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D8" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -587,10 +572,10 @@
         <v>13</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -601,66 +586,10 @@
         <v>14</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" t="s">
-        <v>5</v>
-      </c>
-      <c r="B11" t="s">
-        <v>15</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" t="s">
-        <v>5</v>
-      </c>
-      <c r="B12" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D12" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="A13" t="s">
-        <v>5</v>
-      </c>
-      <c r="B13" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D13" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" t="s">
-        <v>5</v>
-      </c>
-      <c r="B14" t="s">
-        <v>18</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D14" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -674,10 +603,6 @@
     <hyperlink ref="C8" r:id="rId7"/>
     <hyperlink ref="C9" r:id="rId8"/>
     <hyperlink ref="C10" r:id="rId9"/>
-    <hyperlink ref="C11" r:id="rId10"/>
-    <hyperlink ref="C12" r:id="rId11"/>
-    <hyperlink ref="C13" r:id="rId12"/>
-    <hyperlink ref="C14" r:id="rId13"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Validated report update 2025-11-08 19:02
</commit_message>
<xml_diff>
--- a/flagged_segments.xlsx
+++ b/flagged_segments.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="20">
   <si>
     <t>Session</t>
   </si>
@@ -40,25 +40,19 @@
     <t>I'm trying to turn on my kit.</t>
   </si>
   <si>
+    <t>I'm not able to get it to work now.</t>
+  </si>
+  <si>
     <t>I'm not able to… My camera doesn't seem to be working.</t>
   </si>
   <si>
-    <t>You can try restarting my computer.</t>
-  </si>
-  <si>
     <t>… can't… oh, can you hear me?</t>
   </si>
   <si>
-    <t>Yeah, yeah, no, now it's… now it's better. I think the reason I couldn't hear you before is because before I joined the meeting, I didn't click on my headphones, so I was trying to play through my laptop, and it was me.</t>
-  </si>
-  <si>
-    <t>Is it better now?</t>
-  </si>
-  <si>
-    <t>Yeah, the last couple seconds have been okay.</t>
-  </si>
-  <si>
-    <t>What do you think is this… what do you think does this energy makeup look like for reactions that are actually reversible and not complete reactions like this one?</t>
+    <t>Hello?</t>
+  </si>
+  <si>
+    <t>It's unfair to you if we just go on like this for the next 30, 40 minutes of this session. If the internet issue continues happening, then I'll just ask them to, like, not charge you for the session. Hello? Can you hear me?</t>
   </si>
   <si>
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20251026-075624_validated_report.html</t>
@@ -74,6 +68,9 @@
   </si>
   <si>
     <t>Technical: Connectivity Issues</t>
+  </si>
+  <si>
+    <t>Administrative: Payment Adjustments</t>
   </si>
   <si>
     <t>View Report</t>
@@ -443,7 +440,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -474,10 +471,10 @@
         <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -488,10 +485,10 @@
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -502,10 +499,10 @@
         <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -516,10 +513,10 @@
         <v>9</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -530,10 +527,10 @@
         <v>10</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -544,10 +541,10 @@
         <v>11</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -558,38 +555,10 @@
         <v>12</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D8" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" t="s">
-        <v>5</v>
-      </c>
-      <c r="B10" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -601,8 +570,6 @@
     <hyperlink ref="C6" r:id="rId5"/>
     <hyperlink ref="C7" r:id="rId6"/>
     <hyperlink ref="C8" r:id="rId7"/>
-    <hyperlink ref="C9" r:id="rId8"/>
-    <hyperlink ref="C10" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Validated report update 2025-11-08 19:06
</commit_message>
<xml_diff>
--- a/flagged_segments.xlsx
+++ b/flagged_segments.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="29">
   <si>
     <t>Session</t>
   </si>
@@ -37,24 +37,51 @@
     <t>Yeah, I'm here, but I cannot see you.</t>
   </si>
   <si>
-    <t>I'm trying to turn on my kit.</t>
-  </si>
-  <si>
-    <t>I'm not able to get it to work now.</t>
-  </si>
-  <si>
     <t>I'm not able to… My camera doesn't seem to be working.</t>
   </si>
   <si>
-    <t>… can't… oh, can you hear me?</t>
-  </si>
-  <si>
-    <t>Hello?</t>
+    <t>They make it seem like it's so complicated, but really? Turn it off and turn it on. It's like a light switch.</t>
+  </si>
+  <si>
+    <t>Yes?</t>
+  </si>
+  <si>
+    <t>I have no time in my schedule for anything, right?</t>
+  </si>
+  <si>
+    <t>Yeah, and so now you're… when you're seeing… if you could tell me what mercantilism is… what is that again? Do you remember?</t>
+  </si>
+  <si>
+    <t>Right, when we're talking about land-based empires?</t>
+  </si>
+  <si>
+    <t>Right? So, when I say it from that point of view, you're like, yeah, of course that makes sense.</t>
+  </si>
+  <si>
+    <t>Hi, can you hear me?</t>
+  </si>
+  <si>
+    <t>Nope.</t>
+  </si>
+  <si>
+    <t>Can you hear me?</t>
+  </si>
+  <si>
+    <t>Yeah, I can hear you, Vuz, it's just really delayed.</t>
+  </si>
+  <si>
+    <t>Yeah, I would make… because you'd be covering things at a quite accelerated rate if you're doing three weeks, 3… 3 sessions a week, so…</t>
   </si>
   <si>
     <t>It's unfair to you if we just go on like this for the next 30, 40 minutes of this session. If the internet issue continues happening, then I'll just ask them to, like, not charge you for the session. Hello? Can you hear me?</t>
   </si>
   <si>
+    <t>Hello.</t>
+  </si>
+  <si>
+    <t>Yeah, yeah, okay, because I don't think, …</t>
+  </si>
+  <si>
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20251026-075624_validated_report.html</t>
   </si>
   <si>
@@ -64,10 +91,10 @@
     <t>Technical: Video Issues</t>
   </si>
   <si>
+    <t>Technical: Connectivity Issues</t>
+  </si>
+  <si>
     <t>Technical: Audio Issues</t>
-  </si>
-  <si>
-    <t>Technical: Connectivity Issues</t>
   </si>
   <si>
     <t>Administrative: Payment Adjustments</t>
@@ -440,7 +467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -471,10 +498,10 @@
         <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -485,10 +512,10 @@
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="D3" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -499,10 +526,10 @@
         <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -513,52 +540,178 @@
         <v>9</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="D5" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" t="s">
         <v>10</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="D6" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="D7" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B8" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D13" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B15" t="s">
         <v>19</v>
       </c>
-      <c r="D8" t="s">
-        <v>18</v>
+      <c r="C15" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D15" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D16" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" t="s">
+        <v>5</v>
+      </c>
+      <c r="B17" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D17" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -570,6 +723,15 @@
     <hyperlink ref="C6" r:id="rId5"/>
     <hyperlink ref="C7" r:id="rId6"/>
     <hyperlink ref="C8" r:id="rId7"/>
+    <hyperlink ref="C9" r:id="rId8"/>
+    <hyperlink ref="C10" r:id="rId9"/>
+    <hyperlink ref="C11" r:id="rId10"/>
+    <hyperlink ref="C12" r:id="rId11"/>
+    <hyperlink ref="C13" r:id="rId12"/>
+    <hyperlink ref="C14" r:id="rId13"/>
+    <hyperlink ref="C15" r:id="rId14"/>
+    <hyperlink ref="C16" r:id="rId15"/>
+    <hyperlink ref="C17" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Validated report update 2025-11-08 19:09
</commit_message>
<xml_diff>
--- a/flagged_segments.xlsx
+++ b/flagged_segments.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="32">
   <si>
     <t>Session</t>
   </si>
@@ -34,52 +34,58 @@
     <t>GMT20250821-130122</t>
   </si>
   <si>
+    <t>Ram?</t>
+  </si>
+  <si>
     <t>Yeah, I'm here, but I cannot see you.</t>
   </si>
   <si>
     <t>I'm not able to… My camera doesn't seem to be working.</t>
   </si>
   <si>
-    <t>They make it seem like it's so complicated, but really? Turn it off and turn it on. It's like a light switch.</t>
-  </si>
-  <si>
-    <t>Yes?</t>
-  </si>
-  <si>
-    <t>I have no time in my schedule for anything, right?</t>
-  </si>
-  <si>
-    <t>Yeah, and so now you're… when you're seeing… if you could tell me what mercantilism is… what is that again? Do you remember?</t>
-  </si>
-  <si>
-    <t>Right, when we're talking about land-based empires?</t>
-  </si>
-  <si>
-    <t>Right? So, when I say it from that point of view, you're like, yeah, of course that makes sense.</t>
-  </si>
-  <si>
-    <t>Hi, can you hear me?</t>
-  </si>
-  <si>
-    <t>Nope.</t>
-  </si>
-  <si>
-    <t>Can you hear me?</t>
+    <t>Okay, I saw you before, so, it…</t>
+  </si>
+  <si>
+    <t>Yeah. And something as basic as turning it off and turning it on again can find solutions.</t>
+  </si>
+  <si>
+    <t>Mostly, yeah.</t>
+  </si>
+  <si>
+    <t>Yeah, which was… sounds astounding, because…</t>
+  </si>
+  <si>
+    <t>I think they developed gunpowder, like, weapons, like cannons.</t>
+  </si>
+  <si>
+    <t>It's kind of important to note, because geographically, they're sort of in the same… it's Mecca and Medina, right?</t>
+  </si>
+  <si>
+    <t>Hello, can you hear me? I can hear you.</t>
   </si>
   <si>
     <t>Yeah, I can hear you, Vuz, it's just really delayed.</t>
   </si>
   <si>
-    <t>Yeah, I would make… because you'd be covering things at a quite accelerated rate if you're doing three weeks, 3… 3 sessions a week, so…</t>
-  </si>
-  <si>
-    <t>It's unfair to you if we just go on like this for the next 30, 40 minutes of this session. If the internet issue continues happening, then I'll just ask them to, like, not charge you for the session. Hello? Can you hear me?</t>
-  </si>
-  <si>
-    <t>Hello.</t>
-  </si>
-  <si>
-    <t>Yeah, yeah, okay, because I don't think, …</t>
+    <t>Yeah, I can hear you fine.</t>
+  </si>
+  <si>
+    <t>I am definitely lagging. Or, or I don't know, there's something off.</t>
+  </si>
+  <si>
+    <t>….</t>
+  </si>
+  <si>
+    <t>5 to 10 minutes. I will have to leave by, like, 3 sharp, so I'm really sorry about that. But we can definitely stay on longer next week, because I don't have a meeting right after our session, because usually we meet at 4. Does that work?</t>
+  </si>
+  <si>
+    <t>So, what I'm saying is, I'll ask the team to cancel the session from our end.</t>
+  </si>
+  <si>
+    <t>I am writing. Maybe it'll appear for you on a… in a bit, I'm not sure.</t>
+  </si>
+  <si>
+    <t>Okay, thank you.</t>
   </si>
   <si>
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20251026-075624_validated_report.html</t>
@@ -88,16 +94,19 @@
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20250821-130122_validated_report.html</t>
   </si>
   <si>
+    <t>Technical: Connectivity Issues</t>
+  </si>
+  <si>
     <t>Technical: Video Issues</t>
   </si>
   <si>
-    <t>Technical: Connectivity Issues</t>
-  </si>
-  <si>
     <t>Technical: Audio Issues</t>
   </si>
   <si>
-    <t>Administrative: Payment Adjustments</t>
+    <t>Technical: Screen Sharing Problems</t>
+  </si>
+  <si>
+    <t>Administrative: Session Cancellation / Rescheduling</t>
   </si>
   <si>
     <t>View Report</t>
@@ -467,7 +476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -498,10 +507,10 @@
         <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -512,10 +521,10 @@
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D3" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -526,10 +535,10 @@
         <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -540,10 +549,10 @@
         <v>9</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -554,10 +563,10 @@
         <v>10</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -568,10 +577,10 @@
         <v>11</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -582,10 +591,10 @@
         <v>12</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -596,24 +605,24 @@
         <v>13</v>
       </c>
       <c r="C9" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" t="s">
         <v>28</v>
-      </c>
-      <c r="D9" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B10" t="s">
         <v>14</v>
       </c>
       <c r="C10" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" t="s">
         <v>28</v>
-      </c>
-      <c r="D10" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -624,10 +633,10 @@
         <v>15</v>
       </c>
       <c r="C11" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D11" t="s">
         <v>28</v>
-      </c>
-      <c r="D11" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -638,7 +647,7 @@
         <v>16</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D12" t="s">
         <v>26</v>
@@ -652,10 +661,10 @@
         <v>17</v>
       </c>
       <c r="C13" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" t="s">
         <v>28</v>
-      </c>
-      <c r="D13" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -666,10 +675,10 @@
         <v>18</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D14" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -680,10 +689,10 @@
         <v>19</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -694,10 +703,10 @@
         <v>20</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D16" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -708,10 +717,38 @@
         <v>21</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D17" t="s">
-        <v>27</v>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" t="s">
+        <v>5</v>
+      </c>
+      <c r="B18" t="s">
+        <v>22</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D18" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" t="s">
+        <v>5</v>
+      </c>
+      <c r="B19" t="s">
+        <v>23</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D19" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -732,6 +769,8 @@
     <hyperlink ref="C15" r:id="rId14"/>
     <hyperlink ref="C16" r:id="rId15"/>
     <hyperlink ref="C17" r:id="rId16"/>
+    <hyperlink ref="C18" r:id="rId17"/>
+    <hyperlink ref="C19" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Validated report update 2025-11-08 19:20
</commit_message>
<xml_diff>
--- a/flagged_segments.xlsx
+++ b/flagged_segments.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="38">
   <si>
     <t>Session</t>
   </si>
@@ -34,58 +34,79 @@
     <t>GMT20250821-130122</t>
   </si>
   <si>
-    <t>Ram?</t>
-  </si>
-  <si>
     <t>Yeah, I'm here, but I cannot see you.</t>
   </si>
   <si>
     <t>I'm not able to… My camera doesn't seem to be working.</t>
   </si>
   <si>
-    <t>Okay, I saw you before, so, it…</t>
-  </si>
-  <si>
-    <t>Yeah. And something as basic as turning it off and turning it on again can find solutions.</t>
-  </si>
-  <si>
-    <t>Mostly, yeah.</t>
-  </si>
-  <si>
-    <t>Yeah, which was… sounds astounding, because…</t>
-  </si>
-  <si>
-    <t>I think they developed gunpowder, like, weapons, like cannons.</t>
-  </si>
-  <si>
-    <t>It's kind of important to note, because geographically, they're sort of in the same… it's Mecca and Medina, right?</t>
-  </si>
-  <si>
-    <t>Hello, can you hear me? I can hear you.</t>
+    <t>Yeah.</t>
+  </si>
+  <si>
+    <t>Isn't it weird how that, technology can be, like, a little bit fickle?</t>
+  </si>
+  <si>
+    <t>Maybe not always, but, a lot. Okay.</t>
+  </si>
+  <si>
+    <t>I mean, on Tuesday, so…</t>
+  </si>
+  <si>
+    <t>Right? But they, they were stuck.</t>
+  </si>
+  <si>
+    <t>Hello!</t>
+  </si>
+  <si>
+    <t>Hi, can you hear me?</t>
+  </si>
+  <si>
+    <t>Nope.</t>
+  </si>
+  <si>
+    <t>I can, yeah, but can you hear me?</t>
+  </si>
+  <si>
+    <t>Oh, interesting. I'll double-check my audio, but I think… oh, you can't hear me, one second.</t>
+  </si>
+  <si>
+    <t>Hello? I don't know if you can hear me, but I'll leave the call and just join back.</t>
   </si>
   <si>
     <t>Yeah, I can hear you, Vuz, it's just really delayed.</t>
   </si>
   <si>
-    <t>Yeah, I can hear you fine.</t>
+    <t>Is it better now?</t>
+  </si>
+  <si>
+    <t>Okay, can you hear me properly, by the way?</t>
   </si>
   <si>
     <t>I am definitely lagging. Or, or I don't know, there's something off.</t>
   </si>
   <si>
-    <t>….</t>
+    <t>Hello? Oh my god, I'm… I don't know what's happening. …</t>
   </si>
   <si>
     <t>5 to 10 minutes. I will have to leave by, like, 3 sharp, so I'm really sorry about that. But we can definitely stay on longer next week, because I don't have a meeting right after our session, because usually we meet at 4. Does that work?</t>
   </si>
   <si>
+    <t>Yeah, I think it's delayed.</t>
+  </si>
+  <si>
+    <t>Hello. Oh god.</t>
+  </si>
+  <si>
     <t>So, what I'm saying is, I'll ask the team to cancel the session from our end.</t>
   </si>
   <si>
-    <t>I am writing. Maybe it'll appear for you on a… in a bit, I'm not sure.</t>
-  </si>
-  <si>
-    <t>Okay, thank you.</t>
+    <t>Is that fine? I think it's just unfair to you that I just talk and you spend, like, half the time deciphering what I'm saying because of internet issues.</t>
+  </si>
+  <si>
+    <t>then, we're good, and then I'll make that 30 minutes up for you, and, like, either a free session, or we can just add it to the next session, without you being charged for it.</t>
+  </si>
+  <si>
+    <t>Yeah, but I feel bad just because it wasn't the most efficient 40 minutes. Maybe we can just add a little more time, like, I can stay on for a little longer during our next session, just to kind of make sure that everything we covered today is</t>
   </si>
   <si>
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20251026-075624_validated_report.html</t>
@@ -94,16 +115,13 @@
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20250821-130122_validated_report.html</t>
   </si>
   <si>
+    <t>Technical: Video Issues</t>
+  </si>
+  <si>
     <t>Technical: Connectivity Issues</t>
   </si>
   <si>
-    <t>Technical: Video Issues</t>
-  </si>
-  <si>
     <t>Technical: Audio Issues</t>
-  </si>
-  <si>
-    <t>Technical: Screen Sharing Problems</t>
   </si>
   <si>
     <t>Administrative: Session Cancellation / Rescheduling</t>
@@ -476,7 +494,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -507,10 +525,10 @@
         <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D2" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -521,10 +539,10 @@
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D3" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -535,10 +553,10 @@
         <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D4" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -549,10 +567,10 @@
         <v>9</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -563,10 +581,10 @@
         <v>10</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D6" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -577,10 +595,10 @@
         <v>11</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D7" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -591,38 +609,38 @@
         <v>12</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D8" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B9" t="s">
         <v>13</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D9" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B10" t="s">
         <v>14</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D10" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -633,10 +651,10 @@
         <v>15</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D11" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -647,10 +665,10 @@
         <v>16</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D12" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -661,10 +679,10 @@
         <v>17</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D13" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -675,10 +693,10 @@
         <v>18</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D14" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -689,10 +707,10 @@
         <v>19</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D15" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -703,10 +721,10 @@
         <v>20</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D16" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -717,10 +735,10 @@
         <v>21</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D17" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -731,10 +749,10 @@
         <v>22</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D18" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -745,10 +763,108 @@
         <v>23</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D19" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" t="s">
+        <v>5</v>
+      </c>
+      <c r="B20" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D20" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" t="s">
+        <v>5</v>
+      </c>
+      <c r="B21" t="s">
+        <v>25</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D21" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" t="s">
+        <v>5</v>
+      </c>
+      <c r="B22" t="s">
+        <v>26</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D22" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" t="s">
+        <v>5</v>
+      </c>
+      <c r="B23" t="s">
+        <v>27</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D23" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B24" t="s">
+        <v>28</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D24" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" t="s">
+        <v>5</v>
+      </c>
+      <c r="B25" t="s">
+        <v>29</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D25" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" t="s">
+        <v>5</v>
+      </c>
+      <c r="B26" t="s">
         <v>30</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D26" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -771,6 +887,13 @@
     <hyperlink ref="C17" r:id="rId16"/>
     <hyperlink ref="C18" r:id="rId17"/>
     <hyperlink ref="C19" r:id="rId18"/>
+    <hyperlink ref="C20" r:id="rId19"/>
+    <hyperlink ref="C21" r:id="rId20"/>
+    <hyperlink ref="C22" r:id="rId21"/>
+    <hyperlink ref="C23" r:id="rId22"/>
+    <hyperlink ref="C24" r:id="rId23"/>
+    <hyperlink ref="C25" r:id="rId24"/>
+    <hyperlink ref="C26" r:id="rId25"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Validated report update 2025-11-08 19:22
</commit_message>
<xml_diff>
--- a/flagged_segments.xlsx
+++ b/flagged_segments.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="37">
   <si>
     <t>Session</t>
   </si>
@@ -37,22 +37,19 @@
     <t>Yeah, I'm here, but I cannot see you.</t>
   </si>
   <si>
+    <t>I'm not able to get it to work now.</t>
+  </si>
+  <si>
     <t>I'm not able to… My camera doesn't seem to be working.</t>
   </si>
   <si>
-    <t>Yeah.</t>
-  </si>
-  <si>
-    <t>Isn't it weird how that, technology can be, like, a little bit fickle?</t>
-  </si>
-  <si>
-    <t>Maybe not always, but, a lot. Okay.</t>
-  </si>
-  <si>
-    <t>I mean, on Tuesday, so…</t>
-  </si>
-  <si>
-    <t>Right? But they, they were stuck.</t>
+    <t>There should be…</t>
+  </si>
+  <si>
+    <t>I'm in 10th grade.</t>
+  </si>
+  <si>
+    <t>You don't use that… that terminology?</t>
   </si>
   <si>
     <t>Hello!</t>
@@ -64,49 +61,37 @@
     <t>Nope.</t>
   </si>
   <si>
-    <t>I can, yeah, but can you hear me?</t>
-  </si>
-  <si>
     <t>Oh, interesting. I'll double-check my audio, but I think… oh, you can't hear me, one second.</t>
   </si>
   <si>
-    <t>Hello? I don't know if you can hear me, but I'll leave the call and just join back.</t>
-  </si>
-  <si>
-    <t>Yeah, I can hear you, Vuz, it's just really delayed.</t>
-  </si>
-  <si>
-    <t>Is it better now?</t>
-  </si>
-  <si>
-    <t>Okay, can you hear me properly, by the way?</t>
-  </si>
-  <si>
-    <t>I am definitely lagging. Or, or I don't know, there's something off.</t>
-  </si>
-  <si>
-    <t>Hello? Oh my god, I'm… I don't know what's happening. …</t>
-  </si>
-  <si>
-    <t>5 to 10 minutes. I will have to leave by, like, 3 sharp, so I'm really sorry about that. But we can definitely stay on longer next week, because I don't have a meeting right after our session, because usually we meet at 4. Does that work?</t>
-  </si>
-  <si>
-    <t>Yeah, I think it's delayed.</t>
-  </si>
-  <si>
-    <t>Hello. Oh god.</t>
-  </si>
-  <si>
-    <t>So, what I'm saying is, I'll ask the team to cancel the session from our end.</t>
-  </si>
-  <si>
-    <t>Is that fine? I think it's just unfair to you that I just talk and you spend, like, half the time deciphering what I'm saying because of internet issues.</t>
-  </si>
-  <si>
-    <t>then, we're good, and then I'll make that 30 minutes up for you, and, like, either a free session, or we can just add it to the next session, without you being charged for it.</t>
-  </si>
-  <si>
-    <t>Yeah, but I feel bad just because it wasn't the most efficient 40 minutes. Maybe we can just add a little more time, like, I can stay on for a little longer during our next session, just to kind of make sure that everything we covered today is</t>
+    <t>Gotcha. I think my Wi-Fi should be fine.</t>
+  </si>
+  <si>
+    <t>Yeah, I would make… because you'd be covering things at a quite accelerated rate if you're doing three weeks, 3… 3 sessions a week, so…</t>
+  </si>
+  <si>
+    <t>How do we define stability in chemistry?</t>
+  </si>
+  <si>
+    <t>There's, like, slight cuts of….</t>
+  </si>
+  <si>
+    <t>Wi-Fi or yours. Give me just a second, I'll try to restart my Wi-Fi very quickly.</t>
+  </si>
+  <si>
+    <t>Hello?</t>
+  </si>
+  <si>
+    <t>I think it's not from this end, because my wife and I are showing that everything.</t>
+  </si>
+  <si>
+    <t>plus H2….</t>
+  </si>
+  <si>
+    <t>I'd rather I ask them… I know it's… it has been a waste of time for you and for me, but I… I'm totally fine with them canceling the class, and not charging you for it, just because, honestly, I don't think</t>
+  </si>
+  <si>
+    <t>two things in total. So… so yeah, I'll ask them to cancel it, and then hopefully they can contact you to figure out a time for a makeup class.</t>
   </si>
   <si>
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20251026-075624_validated_report.html</t>
@@ -118,10 +103,22 @@
     <t>Technical: Video Issues</t>
   </si>
   <si>
+    <t>Student Behavior Issues: Homework Non-Completion</t>
+  </si>
+  <si>
+    <t>Session Quality: Lack of Engagement</t>
+  </si>
+  <si>
+    <t>Technical: Audio Issues</t>
+  </si>
+  <si>
     <t>Technical: Connectivity Issues</t>
   </si>
   <si>
-    <t>Technical: Audio Issues</t>
+    <t>Administrative: Payment Adjustments</t>
+  </si>
+  <si>
+    <t>Technical: Screen Sharing Problems</t>
   </si>
   <si>
     <t>Administrative: Session Cancellation / Rescheduling</t>
@@ -494,7 +491,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -525,10 +522,10 @@
         <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D2" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -539,10 +536,10 @@
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D3" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -553,10 +550,10 @@
         <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -567,10 +564,10 @@
         <v>9</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D5" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -581,10 +578,10 @@
         <v>10</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -595,24 +592,24 @@
         <v>11</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B8" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D8" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -623,10 +620,10 @@
         <v>13</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D9" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -637,10 +634,10 @@
         <v>14</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -651,10 +648,10 @@
         <v>15</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D11" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -665,10 +662,10 @@
         <v>16</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D12" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -679,10 +676,10 @@
         <v>17</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D13" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -693,10 +690,10 @@
         <v>18</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D14" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -707,10 +704,10 @@
         <v>19</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D15" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -721,10 +718,10 @@
         <v>20</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D16" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -735,10 +732,10 @@
         <v>21</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D17" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -749,10 +746,10 @@
         <v>22</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D18" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -763,7 +760,7 @@
         <v>23</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D19" t="s">
         <v>34</v>
@@ -777,10 +774,10 @@
         <v>24</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D20" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -791,80 +788,10 @@
         <v>25</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D21" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4">
-      <c r="A22" t="s">
-        <v>5</v>
-      </c>
-      <c r="B22" t="s">
-        <v>26</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D22" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4">
-      <c r="A23" t="s">
-        <v>5</v>
-      </c>
-      <c r="B23" t="s">
-        <v>27</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D23" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4">
-      <c r="A24" t="s">
-        <v>5</v>
-      </c>
-      <c r="B24" t="s">
-        <v>28</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D24" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4">
-      <c r="A25" t="s">
-        <v>5</v>
-      </c>
-      <c r="B25" t="s">
-        <v>29</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D25" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4">
-      <c r="A26" t="s">
-        <v>5</v>
-      </c>
-      <c r="B26" t="s">
-        <v>30</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D26" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -889,11 +816,6 @@
     <hyperlink ref="C19" r:id="rId18"/>
     <hyperlink ref="C20" r:id="rId19"/>
     <hyperlink ref="C21" r:id="rId20"/>
-    <hyperlink ref="C22" r:id="rId21"/>
-    <hyperlink ref="C23" r:id="rId22"/>
-    <hyperlink ref="C24" r:id="rId23"/>
-    <hyperlink ref="C25" r:id="rId24"/>
-    <hyperlink ref="C26" r:id="rId25"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Validated report update 2025-11-08 19:24
</commit_message>
<xml_diff>
--- a/flagged_segments.xlsx
+++ b/flagged_segments.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="33">
   <si>
     <t>Session</t>
   </si>
@@ -43,13 +43,22 @@
     <t>I'm not able to… My camera doesn't seem to be working.</t>
   </si>
   <si>
-    <t>There should be…</t>
-  </si>
-  <si>
-    <t>I'm in 10th grade.</t>
-  </si>
-  <si>
-    <t>You don't use that… that terminology?</t>
+    <t>Just try that.</t>
+  </si>
+  <si>
+    <t>Yeah. And something as basic as turning it off and turning it on again can find solutions.</t>
+  </si>
+  <si>
+    <t>Yeah, you literally are just on Unit 3. You have just finished Unit 3.</t>
+  </si>
+  <si>
+    <t>Articles, videos, whatever it may be, to try to give some context into what's going on.</t>
+  </si>
+  <si>
+    <t>No, you don't know, because you haven't started reading it yet.</t>
+  </si>
+  <si>
+    <t>That didn't happen, like, right away. You didn't, you didn't open up your phone and find a meme on whatever it might be, and it spreads around the world, and everybody knows about it.</t>
   </si>
   <si>
     <t>Hello!</t>
@@ -58,40 +67,31 @@
     <t>Hi, can you hear me?</t>
   </si>
   <si>
+    <t>… can't… oh, can you hear me?</t>
+  </si>
+  <si>
     <t>Nope.</t>
   </si>
   <si>
-    <t>Oh, interesting. I'll double-check my audio, but I think… oh, you can't hear me, one second.</t>
-  </si>
-  <si>
-    <t>Gotcha. I think my Wi-Fi should be fine.</t>
-  </si>
-  <si>
-    <t>Yeah, I would make… because you'd be covering things at a quite accelerated rate if you're doing three weeks, 3… 3 sessions a week, so…</t>
-  </si>
-  <si>
-    <t>How do we define stability in chemistry?</t>
-  </si>
-  <si>
-    <t>There's, like, slight cuts of….</t>
+    <t>Hello?</t>
+  </si>
+  <si>
+    <t>Yeah, I can hear you, Vuz, it's just really delayed.</t>
+  </si>
+  <si>
+    <t>I am definitely lagging. Or, or I don't know, there's something off.</t>
   </si>
   <si>
     <t>Wi-Fi or yours. Give me just a second, I'll try to restart my Wi-Fi very quickly.</t>
   </si>
   <si>
-    <t>Hello?</t>
-  </si>
-  <si>
-    <t>I think it's not from this end, because my wife and I are showing that everything.</t>
-  </si>
-  <si>
-    <t>plus H2….</t>
-  </si>
-  <si>
-    <t>I'd rather I ask them… I know it's… it has been a waste of time for you and for me, but I… I'm totally fine with them canceling the class, and not charging you for it, just because, honestly, I don't think</t>
-  </si>
-  <si>
-    <t>two things in total. So… so yeah, I'll ask them to cancel it, and then hopefully they can contact you to figure out a time for a makeup class.</t>
+    <t>5 to 10 minutes. I will have to leave by, like, 3 sharp, so I'm really sorry about that. But we can definitely stay on longer next week, because I don't have a meeting right after our session, because usually we meet at 4. Does that work?</t>
+  </si>
+  <si>
+    <t>Yeah, I think it's delayed.</t>
+  </si>
+  <si>
+    <t>Because I think there is a Wi-Fi issue in my department.</t>
   </si>
   <si>
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20251026-075624_validated_report.html</t>
@@ -103,22 +103,10 @@
     <t>Technical: Video Issues</t>
   </si>
   <si>
-    <t>Student Behavior Issues: Homework Non-Completion</t>
-  </si>
-  <si>
-    <t>Session Quality: Lack of Engagement</t>
+    <t>Technical: Connectivity Issues</t>
   </si>
   <si>
     <t>Technical: Audio Issues</t>
-  </si>
-  <si>
-    <t>Technical: Connectivity Issues</t>
-  </si>
-  <si>
-    <t>Administrative: Payment Adjustments</t>
-  </si>
-  <si>
-    <t>Technical: Screen Sharing Problems</t>
   </si>
   <si>
     <t>Administrative: Session Cancellation / Rescheduling</t>
@@ -491,7 +479,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -522,7 +510,7 @@
         <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D2" t="s">
         <v>28</v>
@@ -536,7 +524,7 @@
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D3" t="s">
         <v>28</v>
@@ -550,7 +538,7 @@
         <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D4" t="s">
         <v>28</v>
@@ -564,10 +552,10 @@
         <v>9</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -578,7 +566,7 @@
         <v>10</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D6" t="s">
         <v>29</v>
@@ -592,52 +580,52 @@
         <v>11</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B8" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D8" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B9" t="s">
         <v>13</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D9" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B10" t="s">
         <v>14</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D10" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -648,10 +636,10 @@
         <v>15</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -662,10 +650,10 @@
         <v>16</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D12" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -676,10 +664,10 @@
         <v>17</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D13" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -690,10 +678,10 @@
         <v>18</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D14" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -704,10 +692,10 @@
         <v>19</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -715,13 +703,13 @@
         <v>5</v>
       </c>
       <c r="B16" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D16" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -729,13 +717,13 @@
         <v>5</v>
       </c>
       <c r="B17" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D17" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -743,13 +731,13 @@
         <v>5</v>
       </c>
       <c r="B18" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D18" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -757,13 +745,13 @@
         <v>5</v>
       </c>
       <c r="B19" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D19" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -771,13 +759,13 @@
         <v>5</v>
       </c>
       <c r="B20" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D20" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -785,13 +773,55 @@
         <v>5</v>
       </c>
       <c r="B21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D21" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" t="s">
+        <v>5</v>
+      </c>
+      <c r="B22" t="s">
+        <v>24</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D22" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" t="s">
+        <v>5</v>
+      </c>
+      <c r="B23" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D21" t="s">
-        <v>35</v>
+      <c r="C23" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D23" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B24" t="s">
+        <v>19</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D24" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -816,6 +846,9 @@
     <hyperlink ref="C19" r:id="rId18"/>
     <hyperlink ref="C20" r:id="rId19"/>
     <hyperlink ref="C21" r:id="rId20"/>
+    <hyperlink ref="C22" r:id="rId21"/>
+    <hyperlink ref="C23" r:id="rId22"/>
+    <hyperlink ref="C24" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Validated report update 2025-11-08 20:04
</commit_message>
<xml_diff>
--- a/flagged_segments.xlsx
+++ b/flagged_segments.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="20">
   <si>
     <t>Session</t>
   </si>
@@ -40,60 +40,18 @@
     <t>I'm not able to get it to work now.</t>
   </si>
   <si>
-    <t>I'm not able to… My camera doesn't seem to be working.</t>
-  </si>
-  <si>
-    <t>Just try that.</t>
-  </si>
-  <si>
-    <t>Yeah. And something as basic as turning it off and turning it on again can find solutions.</t>
-  </si>
-  <si>
-    <t>Yeah, you literally are just on Unit 3. You have just finished Unit 3.</t>
-  </si>
-  <si>
-    <t>Articles, videos, whatever it may be, to try to give some context into what's going on.</t>
-  </si>
-  <si>
-    <t>No, you don't know, because you haven't started reading it yet.</t>
-  </si>
-  <si>
-    <t>That didn't happen, like, right away. You didn't, you didn't open up your phone and find a meme on whatever it might be, and it spreads around the world, and everybody knows about it.</t>
-  </si>
-  <si>
-    <t>Hello!</t>
+    <t>An American system is called freshman, sophomore, junior, senior.</t>
+  </si>
+  <si>
+    <t>education included, right? So if there is, then it's probably an underground society.</t>
+  </si>
+  <si>
+    <t>Well, kind of, but…</t>
   </si>
   <si>
     <t>Hi, can you hear me?</t>
   </si>
   <si>
-    <t>… can't… oh, can you hear me?</t>
-  </si>
-  <si>
-    <t>Nope.</t>
-  </si>
-  <si>
-    <t>Hello?</t>
-  </si>
-  <si>
-    <t>Yeah, I can hear you, Vuz, it's just really delayed.</t>
-  </si>
-  <si>
-    <t>I am definitely lagging. Or, or I don't know, there's something off.</t>
-  </si>
-  <si>
-    <t>Wi-Fi or yours. Give me just a second, I'll try to restart my Wi-Fi very quickly.</t>
-  </si>
-  <si>
-    <t>5 to 10 minutes. I will have to leave by, like, 3 sharp, so I'm really sorry about that. But we can definitely stay on longer next week, because I don't have a meeting right after our session, because usually we meet at 4. Does that work?</t>
-  </si>
-  <si>
-    <t>Yeah, I think it's delayed.</t>
-  </si>
-  <si>
-    <t>Because I think there is a Wi-Fi issue in my department.</t>
-  </si>
-  <si>
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20251026-075624_validated_report.html</t>
   </si>
   <si>
@@ -103,13 +61,16 @@
     <t>Technical: Video Issues</t>
   </si>
   <si>
-    <t>Technical: Connectivity Issues</t>
+    <t>Session Quality: Factually Incorrect Information</t>
+  </si>
+  <si>
+    <t>Safety: Illegal Activities</t>
+  </si>
+  <si>
+    <t>Session Quality: Off-Topic Discussion</t>
   </si>
   <si>
     <t>Technical: Audio Issues</t>
-  </si>
-  <si>
-    <t>Administrative: Session Cancellation / Rescheduling</t>
   </si>
   <si>
     <t>View Report</t>
@@ -479,7 +440,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -510,10 +471,10 @@
         <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="D2" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -524,10 +485,10 @@
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="D3" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -538,10 +499,10 @@
         <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="D4" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -552,10 +513,10 @@
         <v>9</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="D5" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -566,262 +527,24 @@
         <v>10</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="D6" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B7" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="D7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" t="s">
-        <v>4</v>
-      </c>
-      <c r="B8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" t="s">
-        <v>4</v>
-      </c>
-      <c r="B9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" t="s">
-        <v>4</v>
-      </c>
-      <c r="B10" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D10" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" t="s">
-        <v>5</v>
-      </c>
-      <c r="B11" t="s">
-        <v>15</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D11" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" t="s">
-        <v>5</v>
-      </c>
-      <c r="B12" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D12" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="A13" t="s">
-        <v>5</v>
-      </c>
-      <c r="B13" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D13" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" t="s">
-        <v>5</v>
-      </c>
-      <c r="B14" t="s">
         <v>18</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D14" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="A15" t="s">
-        <v>5</v>
-      </c>
-      <c r="B15" t="s">
-        <v>19</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D15" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" t="s">
-        <v>5</v>
-      </c>
-      <c r="B16" t="s">
-        <v>19</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D16" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="A17" t="s">
-        <v>5</v>
-      </c>
-      <c r="B17" t="s">
-        <v>20</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D17" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4">
-      <c r="A18" t="s">
-        <v>5</v>
-      </c>
-      <c r="B18" t="s">
-        <v>21</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D18" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4">
-      <c r="A19" t="s">
-        <v>5</v>
-      </c>
-      <c r="B19" t="s">
-        <v>22</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D19" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4">
-      <c r="A20" t="s">
-        <v>5</v>
-      </c>
-      <c r="B20" t="s">
-        <v>23</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D20" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4">
-      <c r="A21" t="s">
-        <v>5</v>
-      </c>
-      <c r="B21" t="s">
-        <v>19</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D21" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4">
-      <c r="A22" t="s">
-        <v>5</v>
-      </c>
-      <c r="B22" t="s">
-        <v>24</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D22" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4">
-      <c r="A23" t="s">
-        <v>5</v>
-      </c>
-      <c r="B23" t="s">
-        <v>25</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D23" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4">
-      <c r="A24" t="s">
-        <v>5</v>
-      </c>
-      <c r="B24" t="s">
-        <v>19</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D24" t="s">
-        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -832,23 +555,6 @@
     <hyperlink ref="C5" r:id="rId4"/>
     <hyperlink ref="C6" r:id="rId5"/>
     <hyperlink ref="C7" r:id="rId6"/>
-    <hyperlink ref="C8" r:id="rId7"/>
-    <hyperlink ref="C9" r:id="rId8"/>
-    <hyperlink ref="C10" r:id="rId9"/>
-    <hyperlink ref="C11" r:id="rId10"/>
-    <hyperlink ref="C12" r:id="rId11"/>
-    <hyperlink ref="C13" r:id="rId12"/>
-    <hyperlink ref="C14" r:id="rId13"/>
-    <hyperlink ref="C15" r:id="rId14"/>
-    <hyperlink ref="C16" r:id="rId15"/>
-    <hyperlink ref="C17" r:id="rId16"/>
-    <hyperlink ref="C18" r:id="rId17"/>
-    <hyperlink ref="C19" r:id="rId18"/>
-    <hyperlink ref="C20" r:id="rId19"/>
-    <hyperlink ref="C21" r:id="rId20"/>
-    <hyperlink ref="C22" r:id="rId21"/>
-    <hyperlink ref="C23" r:id="rId22"/>
-    <hyperlink ref="C24" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Validated report update 2025-11-08 20:06
</commit_message>
<xml_diff>
--- a/flagged_segments.xlsx
+++ b/flagged_segments.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="35">
   <si>
     <t>Session</t>
   </si>
@@ -34,43 +34,88 @@
     <t>GMT20250821-130122</t>
   </si>
   <si>
+    <t>Ram?</t>
+  </si>
+  <si>
+    <t>Hello?</t>
+  </si>
+  <si>
     <t>Yeah, I'm here, but I cannot see you.</t>
   </si>
   <si>
+    <t>I'm not able to… My camera doesn't seem to be working.</t>
+  </si>
+  <si>
     <t>I'm not able to get it to work now.</t>
   </si>
   <si>
-    <t>An American system is called freshman, sophomore, junior, senior.</t>
-  </si>
-  <si>
-    <t>education included, right? So if there is, then it's probably an underground society.</t>
-  </si>
-  <si>
-    <t>Well, kind of, but…</t>
-  </si>
-  <si>
     <t>Hi, can you hear me?</t>
   </si>
   <si>
+    <t>… can't… oh, can you hear me?</t>
+  </si>
+  <si>
+    <t>Nope.</t>
+  </si>
+  <si>
+    <t>Hello, can you hear me? I can hear you.</t>
+  </si>
+  <si>
+    <t>Oh, interesting. I'll double-check my audio, but I think… oh, you can't hear me, one second.</t>
+  </si>
+  <si>
+    <t>Hello? I don't know if you can hear me, but I'll leave the call and just join back.</t>
+  </si>
+  <si>
+    <t>Yeah, I can hear you, Vuz, it's just really delayed.</t>
+  </si>
+  <si>
+    <t>I am definitely lagging. Or, or I don't know, there's something off.</t>
+  </si>
+  <si>
+    <t>Wi-Fi or yours. Give me just a second, I'll try to restart my Wi-Fi very quickly.</t>
+  </si>
+  <si>
+    <t>Oh my god, I'm so sorry, I don't know why. Some meeting rooms… in some meeting rooms in my department, the connection is weird. If I start lagging at any point, let me know again. But yeah, we lost, like.</t>
+  </si>
+  <si>
+    <t>Yeah, yeah. Can you hear me?</t>
+  </si>
+  <si>
+    <t>ask them not to charge you for this class, and then I can give you a full makeup class, instead of this one, because it's unfair to just have you not understand half the things I'm saying.</t>
+  </si>
+  <si>
+    <t>Is that fine? I think it's just unfair to you that I just talk and you spend, like, half the time deciphering what I'm saying because of internet issues.</t>
+  </si>
+  <si>
+    <t>H… H-Lit?</t>
+  </si>
+  <si>
+    <t>Okay.</t>
+  </si>
+  <si>
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20251026-075624_validated_report.html</t>
   </si>
   <si>
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20250821-130122_validated_report.html</t>
   </si>
   <si>
+    <t>Technical: Audio Issues</t>
+  </si>
+  <si>
     <t>Technical: Video Issues</t>
   </si>
   <si>
-    <t>Session Quality: Factually Incorrect Information</t>
-  </si>
-  <si>
-    <t>Safety: Illegal Activities</t>
-  </si>
-  <si>
-    <t>Session Quality: Off-Topic Discussion</t>
-  </si>
-  <si>
-    <t>Technical: Audio Issues</t>
+    <t>Technical: Connectivity Issues</t>
+  </si>
+  <si>
+    <t>Technical: Payment Outside Platform</t>
+  </si>
+  <si>
+    <t>Session Quality: Tutor Monologue</t>
+  </si>
+  <si>
+    <t>Other: Parent Over-Involvement</t>
   </si>
   <si>
     <t>View Report</t>
@@ -440,7 +485,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -471,10 +516,10 @@
         <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="D2" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -485,10 +530,10 @@
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -499,10 +544,10 @@
         <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -513,10 +558,10 @@
         <v>9</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -527,10 +572,10 @@
         <v>10</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="D6" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -541,10 +586,234 @@
         <v>11</v>
       </c>
       <c r="C7" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D12" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D13" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D14" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" t="s">
+        <v>5</v>
+      </c>
+      <c r="B17" t="s">
         <v>19</v>
       </c>
-      <c r="D7" t="s">
-        <v>18</v>
+      <c r="C17" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D17" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" t="s">
+        <v>5</v>
+      </c>
+      <c r="B18" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D18" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" t="s">
+        <v>5</v>
+      </c>
+      <c r="B19" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D19" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" t="s">
+        <v>5</v>
+      </c>
+      <c r="B20" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D20" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" t="s">
+        <v>5</v>
+      </c>
+      <c r="B21" t="s">
+        <v>23</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D21" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" t="s">
+        <v>5</v>
+      </c>
+      <c r="B22" t="s">
+        <v>24</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D22" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" t="s">
+        <v>5</v>
+      </c>
+      <c r="B23" t="s">
+        <v>25</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D23" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -555,6 +824,22 @@
     <hyperlink ref="C5" r:id="rId4"/>
     <hyperlink ref="C6" r:id="rId5"/>
     <hyperlink ref="C7" r:id="rId6"/>
+    <hyperlink ref="C8" r:id="rId7"/>
+    <hyperlink ref="C9" r:id="rId8"/>
+    <hyperlink ref="C10" r:id="rId9"/>
+    <hyperlink ref="C11" r:id="rId10"/>
+    <hyperlink ref="C12" r:id="rId11"/>
+    <hyperlink ref="C13" r:id="rId12"/>
+    <hyperlink ref="C14" r:id="rId13"/>
+    <hyperlink ref="C15" r:id="rId14"/>
+    <hyperlink ref="C16" r:id="rId15"/>
+    <hyperlink ref="C17" r:id="rId16"/>
+    <hyperlink ref="C18" r:id="rId17"/>
+    <hyperlink ref="C19" r:id="rId18"/>
+    <hyperlink ref="C20" r:id="rId19"/>
+    <hyperlink ref="C21" r:id="rId20"/>
+    <hyperlink ref="C22" r:id="rId21"/>
+    <hyperlink ref="C23" r:id="rId22"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Validated report update 2025-11-08 21:04
</commit_message>
<xml_diff>
--- a/flagged_segments.xlsx
+++ b/flagged_segments.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="36">
   <si>
     <t>Session</t>
   </si>
@@ -37,61 +37,61 @@
     <t>Ram?</t>
   </si>
   <si>
+    <t>Yeah, I'm here, but I cannot see you.</t>
+  </si>
+  <si>
+    <t>I'm not able to get it to work now.</t>
+  </si>
+  <si>
+    <t>Sorry.</t>
+  </si>
+  <si>
+    <t>I'm not able to… My camera doesn't seem to be working.</t>
+  </si>
+  <si>
+    <t>They make it seem like it's so complicated, but really? Turn it off and turn it on. It's like a light switch.</t>
+  </si>
+  <si>
+    <t>I know all the information in this book, but this book is only one source.</t>
+  </si>
+  <si>
+    <t>Right? How we use those 24 hours is entirely up to us.</t>
+  </si>
+  <si>
+    <t>Right? In order to get the rewards, you have to be all-in.</t>
+  </si>
+  <si>
+    <t>Getting a bit corrupt?</t>
+  </si>
+  <si>
+    <t>Hi, how are you? Good to see you!</t>
+  </si>
+  <si>
     <t>Hello?</t>
   </si>
   <si>
-    <t>Yeah, I'm here, but I cannot see you.</t>
-  </si>
-  <si>
-    <t>I'm not able to… My camera doesn't seem to be working.</t>
-  </si>
-  <si>
-    <t>I'm not able to get it to work now.</t>
-  </si>
-  <si>
-    <t>Hi, can you hear me?</t>
-  </si>
-  <si>
-    <t>… can't… oh, can you hear me?</t>
-  </si>
-  <si>
-    <t>Nope.</t>
-  </si>
-  <si>
-    <t>Hello, can you hear me? I can hear you.</t>
-  </si>
-  <si>
-    <t>Oh, interesting. I'll double-check my audio, but I think… oh, you can't hear me, one second.</t>
-  </si>
-  <si>
-    <t>Hello? I don't know if you can hear me, but I'll leave the call and just join back.</t>
-  </si>
-  <si>
-    <t>Yeah, I can hear you, Vuz, it's just really delayed.</t>
-  </si>
-  <si>
-    <t>I am definitely lagging. Or, or I don't know, there's something off.</t>
-  </si>
-  <si>
-    <t>Wi-Fi or yours. Give me just a second, I'll try to restart my Wi-Fi very quickly.</t>
-  </si>
-  <si>
-    <t>Oh my god, I'm so sorry, I don't know why. Some meeting rooms… in some meeting rooms in my department, the connection is weird. If I start lagging at any point, let me know again. But yeah, we lost, like.</t>
-  </si>
-  <si>
-    <t>Yeah, yeah. Can you hear me?</t>
-  </si>
-  <si>
-    <t>ask them not to charge you for this class, and then I can give you a full makeup class, instead of this one, because it's unfair to just have you not understand half the things I'm saying.</t>
-  </si>
-  <si>
-    <t>Is that fine? I think it's just unfair to you that I just talk and you spend, like, half the time deciphering what I'm saying because of internet issues.</t>
-  </si>
-  <si>
-    <t>H… H-Lit?</t>
-  </si>
-  <si>
-    <t>Okay.</t>
+    <t>Oh, alright, awesome. Yes, I can hear you, can you hear me?</t>
+  </si>
+  <si>
+    <t>Actually, let me take a step back.</t>
+  </si>
+  <si>
+    <t>I can double-check…</t>
+  </si>
+  <si>
+    <t>5 to 10 minutes. I will have to leave by, like, 3 sharp, so I'm really sorry about that. But we can definitely stay on longer next week, because I don't have a meeting right after our session, because usually we meet at 4. Does that work?</t>
+  </si>
+  <si>
+    <t>It's unfair to you if we just go on like this for the next 30, 40 minutes of this session. If the internet issue continues happening, then I'll just ask them to, like, not charge you for the session. Hello? Can you hear me?</t>
+  </si>
+  <si>
+    <t>So, what I'm saying is, I'll ask the team to cancel the session from our end.</t>
+  </si>
+  <si>
+    <t>Does that make sense?</t>
+  </si>
+  <si>
+    <t>N doesn't seem to be a working.</t>
   </si>
   <si>
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20251026-075624_validated_report.html</t>
@@ -109,13 +109,16 @@
     <t>Technical: Connectivity Issues</t>
   </si>
   <si>
-    <t>Technical: Payment Outside Platform</t>
-  </si>
-  <si>
-    <t>Session Quality: Tutor Monologue</t>
-  </si>
-  <si>
-    <t>Other: Parent Over-Involvement</t>
+    <t>Session Quality: Tutor Knowledge Gaps</t>
+  </si>
+  <si>
+    <t>Session Quality: Lack of Engagement</t>
+  </si>
+  <si>
+    <t>Session Quality: Factually Incorrect Information</t>
+  </si>
+  <si>
+    <t>Technical: Session Cancellation / Rescheduling</t>
   </si>
   <si>
     <t>View Report</t>
@@ -516,7 +519,7 @@
         <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D2" t="s">
         <v>28</v>
@@ -530,10 +533,10 @@
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -544,7 +547,7 @@
         <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D4" t="s">
         <v>29</v>
@@ -558,7 +561,7 @@
         <v>9</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D5" t="s">
         <v>29</v>
@@ -572,80 +575,80 @@
         <v>10</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B8" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D8" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B9" t="s">
         <v>13</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D9" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B10" t="s">
         <v>14</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D10" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B11" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D11" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -653,10 +656,10 @@
         <v>5</v>
       </c>
       <c r="B12" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D12" t="s">
         <v>28</v>
@@ -667,10 +670,10 @@
         <v>5</v>
       </c>
       <c r="B13" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D13" t="s">
         <v>28</v>
@@ -681,10 +684,10 @@
         <v>5</v>
       </c>
       <c r="B14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D14" t="s">
         <v>28</v>
@@ -695,13 +698,13 @@
         <v>5</v>
       </c>
       <c r="B15" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D15" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -709,13 +712,13 @@
         <v>5</v>
       </c>
       <c r="B16" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D16" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -723,10 +726,10 @@
         <v>5</v>
       </c>
       <c r="B17" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D17" t="s">
         <v>30</v>
@@ -740,7 +743,7 @@
         <v>20</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D18" t="s">
         <v>30</v>
@@ -754,10 +757,10 @@
         <v>21</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D19" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -768,10 +771,10 @@
         <v>22</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D20" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -782,10 +785,10 @@
         <v>23</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D21" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -796,10 +799,10 @@
         <v>24</v>
       </c>
       <c r="C22" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D22" t="s">
         <v>34</v>
-      </c>
-      <c r="D22" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -810,10 +813,10 @@
         <v>25</v>
       </c>
       <c r="C23" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D23" t="s">
         <v>34</v>
-      </c>
-      <c r="D23" t="s">
-        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Validated report update 2025-11-08 21:11
</commit_message>
<xml_diff>
--- a/flagged_segments.xlsx
+++ b/flagged_segments.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="31">
   <si>
     <t>Session</t>
   </si>
@@ -34,64 +34,52 @@
     <t>GMT20250821-130122</t>
   </si>
   <si>
-    <t>Ram?</t>
-  </si>
-  <si>
     <t>Yeah, I'm here, but I cannot see you.</t>
   </si>
   <si>
-    <t>I'm not able to get it to work now.</t>
-  </si>
-  <si>
-    <t>Sorry.</t>
-  </si>
-  <si>
     <t>I'm not able to… My camera doesn't seem to be working.</t>
   </si>
   <si>
-    <t>They make it seem like it's so complicated, but really? Turn it off and turn it on. It's like a light switch.</t>
-  </si>
-  <si>
-    <t>I know all the information in this book, but this book is only one source.</t>
-  </si>
-  <si>
-    <t>Right? How we use those 24 hours is entirely up to us.</t>
-  </si>
-  <si>
-    <t>Right? In order to get the rewards, you have to be all-in.</t>
-  </si>
-  <si>
-    <t>Getting a bit corrupt?</t>
-  </si>
-  <si>
-    <t>Hi, how are you? Good to see you!</t>
+    <t>One…</t>
+  </si>
+  <si>
+    <t>Where are you?</t>
   </si>
   <si>
     <t>Hello?</t>
   </si>
   <si>
-    <t>Oh, alright, awesome. Yes, I can hear you, can you hear me?</t>
-  </si>
-  <si>
-    <t>Actually, let me take a step back.</t>
+    <t>Yes?</t>
+  </si>
+  <si>
+    <t>Yeah, sophomore.</t>
+  </si>
+  <si>
+    <t>… can't… oh, can you hear me?</t>
+  </si>
+  <si>
+    <t>Nope.</t>
+  </si>
+  <si>
+    <t>Yeah, I can hear you, Vuz, it's just really delayed.</t>
+  </si>
+  <si>
+    <t>Oh, wow, okay. And do you already have your schedule up for the next academic year?</t>
+  </si>
+  <si>
+    <t>I am definitely lagging. Or, or I don't know, there's something off.</t>
   </si>
   <si>
     <t>I can double-check…</t>
   </si>
   <si>
-    <t>5 to 10 minutes. I will have to leave by, like, 3 sharp, so I'm really sorry about that. But we can definitely stay on longer next week, because I don't have a meeting right after our session, because usually we meet at 4. Does that work?</t>
-  </si>
-  <si>
-    <t>It's unfair to you if we just go on like this for the next 30, 40 minutes of this session. If the internet issue continues happening, then I'll just ask them to, like, not charge you for the session. Hello? Can you hear me?</t>
-  </si>
-  <si>
-    <t>So, what I'm saying is, I'll ask the team to cancel the session from our end.</t>
-  </si>
-  <si>
-    <t>Does that make sense?</t>
-  </si>
-  <si>
-    <t>N doesn't seem to be a working.</t>
+    <t>Is that okay?</t>
+  </si>
+  <si>
+    <t>ask them not to charge you for this class, and then I can give you a full makeup class, instead of this one, because it's unfair to just have you not understand half the things I'm saying.</t>
+  </si>
+  <si>
+    <t>Yes, yes, yeah, I'm just apologizing again, and please also apologize to your parents for me, but we'll make sure to sort this out with the team, and we'll do a makeup class for sure.</t>
   </si>
   <si>
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20251026-075624_validated_report.html</t>
@@ -100,25 +88,22 @@
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20250821-130122_validated_report.html</t>
   </si>
   <si>
+    <t>Technical: Video Issues</t>
+  </si>
+  <si>
     <t>Technical: Audio Issues</t>
   </si>
   <si>
-    <t>Technical: Video Issues</t>
+    <t>Session Quality: Lack of Engagement</t>
   </si>
   <si>
     <t>Technical: Connectivity Issues</t>
   </si>
   <si>
-    <t>Session Quality: Tutor Knowledge Gaps</t>
-  </si>
-  <si>
-    <t>Session Quality: Lack of Engagement</t>
-  </si>
-  <si>
-    <t>Session Quality: Factually Incorrect Information</t>
-  </si>
-  <si>
-    <t>Technical: Session Cancellation / Rescheduling</t>
+    <t>Administrative: Payment Adjustments</t>
+  </si>
+  <si>
+    <t>Administrative: Session Cancellation / Rescheduling</t>
   </si>
   <si>
     <t>View Report</t>
@@ -488,7 +473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -519,10 +504,10 @@
         <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -533,10 +518,10 @@
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D3" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -547,10 +532,10 @@
         <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D4" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -561,10 +546,10 @@
         <v>9</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D5" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -575,10 +560,10 @@
         <v>10</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D6" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -589,10 +574,10 @@
         <v>11</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D7" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -603,52 +588,52 @@
         <v>12</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D8" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B9" t="s">
         <v>13</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D9" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B10" t="s">
         <v>14</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D10" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B11" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D11" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -656,13 +641,13 @@
         <v>5</v>
       </c>
       <c r="B12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -670,13 +655,13 @@
         <v>5</v>
       </c>
       <c r="B13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -687,10 +672,10 @@
         <v>17</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D14" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -701,10 +686,10 @@
         <v>18</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D15" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -715,7 +700,7 @@
         <v>19</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D16" t="s">
         <v>28</v>
@@ -726,13 +711,13 @@
         <v>5</v>
       </c>
       <c r="B17" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D17" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -740,83 +725,13 @@
         <v>5</v>
       </c>
       <c r="B18" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D18" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4">
-      <c r="A19" t="s">
-        <v>5</v>
-      </c>
-      <c r="B19" t="s">
-        <v>21</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D19" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4">
-      <c r="A20" t="s">
-        <v>5</v>
-      </c>
-      <c r="B20" t="s">
-        <v>22</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D20" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4">
-      <c r="A21" t="s">
-        <v>5</v>
-      </c>
-      <c r="B21" t="s">
-        <v>23</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D21" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4">
-      <c r="A22" t="s">
-        <v>5</v>
-      </c>
-      <c r="B22" t="s">
-        <v>24</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D22" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4">
-      <c r="A23" t="s">
-        <v>5</v>
-      </c>
-      <c r="B23" t="s">
-        <v>25</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D23" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -838,11 +753,6 @@
     <hyperlink ref="C16" r:id="rId15"/>
     <hyperlink ref="C17" r:id="rId16"/>
     <hyperlink ref="C18" r:id="rId17"/>
-    <hyperlink ref="C19" r:id="rId18"/>
-    <hyperlink ref="C20" r:id="rId19"/>
-    <hyperlink ref="C21" r:id="rId20"/>
-    <hyperlink ref="C22" r:id="rId21"/>
-    <hyperlink ref="C23" r:id="rId22"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Validated report update 2025-11-08 21:18
</commit_message>
<xml_diff>
--- a/flagged_segments.xlsx
+++ b/flagged_segments.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="36">
   <si>
     <t>Session</t>
   </si>
@@ -34,52 +34,61 @@
     <t>GMT20250821-130122</t>
   </si>
   <si>
+    <t>Hello?</t>
+  </si>
+  <si>
     <t>Yeah, I'm here, but I cannot see you.</t>
   </si>
   <si>
-    <t>I'm not able to… My camera doesn't seem to be working.</t>
-  </si>
-  <si>
-    <t>One…</t>
-  </si>
-  <si>
-    <t>Where are you?</t>
-  </si>
-  <si>
-    <t>Hello?</t>
-  </si>
-  <si>
-    <t>Yes?</t>
+    <t>I'm not able to get it to work now.</t>
+  </si>
+  <si>
+    <t>Sorry.</t>
+  </si>
+  <si>
+    <t>You can try restarting my computer.</t>
+  </si>
+  <si>
+    <t>It's scary, because… If that's how things really work, And we've all been fooled.</t>
   </si>
   <si>
     <t>Yeah, sophomore.</t>
   </si>
   <si>
+    <t>We certainly know that religion is being stifled, now, in China.</t>
+  </si>
+  <si>
+    <t>What's that, race called again? The…</t>
+  </si>
+  <si>
+    <t>Hi, can you hear me?</t>
+  </si>
+  <si>
     <t>… can't… oh, can you hear me?</t>
   </si>
   <si>
     <t>Nope.</t>
   </si>
   <si>
-    <t>Yeah, I can hear you, Vuz, it's just really delayed.</t>
-  </si>
-  <si>
-    <t>Oh, wow, okay. And do you already have your schedule up for the next academic year?</t>
+    <t>Oh, interesting. I'll double-check my audio, but I think… oh, you can't hear me, one second.</t>
+  </si>
+  <si>
+    <t>Not, not yet.</t>
   </si>
   <si>
     <t>I am definitely lagging. Or, or I don't know, there's something off.</t>
   </si>
   <si>
-    <t>I can double-check…</t>
-  </si>
-  <si>
-    <t>Is that okay?</t>
-  </si>
-  <si>
-    <t>ask them not to charge you for this class, and then I can give you a full makeup class, instead of this one, because it's unfair to just have you not understand half the things I'm saying.</t>
-  </si>
-  <si>
-    <t>Yes, yes, yeah, I'm just apologizing again, and please also apologize to your parents for me, but we'll make sure to sort this out with the team, and we'll do a makeup class for sure.</t>
+    <t>then let me know, I can try my best to…</t>
+  </si>
+  <si>
+    <t>5 to 10 minutes. I will have to leave by, like, 3 sharp, so I'm really sorry about that. But we can definitely stay on longer next week, because I don't have a meeting right after our session, because usually we meet at 4. Does that work?</t>
+  </si>
+  <si>
+    <t>Hello.</t>
+  </si>
+  <si>
+    <t>I can.</t>
   </si>
   <si>
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20251026-075624_validated_report.html</t>
@@ -88,22 +97,28 @@
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20250821-130122_validated_report.html</t>
   </si>
   <si>
+    <t>Technical: Audio Issues</t>
+  </si>
+  <si>
     <t>Technical: Video Issues</t>
   </si>
   <si>
-    <t>Technical: Audio Issues</t>
+    <t>Technical: Connectivity Issues</t>
+  </si>
+  <si>
+    <t>Session Quality: Off-Topic Discussion</t>
   </si>
   <si>
     <t>Session Quality: Lack of Engagement</t>
   </si>
   <si>
-    <t>Technical: Connectivity Issues</t>
+    <t>Session Quality: Not Understanding the Material</t>
   </si>
   <si>
     <t>Administrative: Payment Adjustments</t>
   </si>
   <si>
-    <t>Administrative: Session Cancellation / Rescheduling</t>
+    <t>Technical: Screen Sharing Problems</t>
   </si>
   <si>
     <t>View Report</t>
@@ -473,7 +488,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -504,10 +519,10 @@
         <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -518,10 +533,10 @@
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -532,10 +547,10 @@
         <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -546,10 +561,10 @@
         <v>9</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -560,10 +575,10 @@
         <v>10</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -574,10 +589,10 @@
         <v>11</v>
       </c>
       <c r="C7" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" t="s">
         <v>30</v>
-      </c>
-      <c r="D7" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -588,38 +603,38 @@
         <v>12</v>
       </c>
       <c r="C8" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" t="s">
         <v>30</v>
-      </c>
-      <c r="D8" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B9" t="s">
         <v>13</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D9" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B10" t="s">
         <v>14</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D10" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -627,13 +642,13 @@
         <v>5</v>
       </c>
       <c r="B11" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D11" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -641,10 +656,10 @@
         <v>5</v>
       </c>
       <c r="B12" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D12" t="s">
         <v>27</v>
@@ -655,10 +670,10 @@
         <v>5</v>
       </c>
       <c r="B13" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D13" t="s">
         <v>27</v>
@@ -669,10 +684,10 @@
         <v>5</v>
       </c>
       <c r="B14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D14" t="s">
         <v>27</v>
@@ -683,13 +698,13 @@
         <v>5</v>
       </c>
       <c r="B15" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -697,13 +712,13 @@
         <v>5</v>
       </c>
       <c r="B16" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D16" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -711,13 +726,13 @@
         <v>5</v>
       </c>
       <c r="B17" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D17" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -725,13 +740,41 @@
         <v>5</v>
       </c>
       <c r="B18" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D18" t="s">
-        <v>29</v>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" t="s">
+        <v>5</v>
+      </c>
+      <c r="B19" t="s">
+        <v>23</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D19" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" t="s">
+        <v>5</v>
+      </c>
+      <c r="B20" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D20" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -753,6 +796,8 @@
     <hyperlink ref="C16" r:id="rId15"/>
     <hyperlink ref="C17" r:id="rId16"/>
     <hyperlink ref="C18" r:id="rId17"/>
+    <hyperlink ref="C19" r:id="rId18"/>
+    <hyperlink ref="C20" r:id="rId19"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Validated report update 2025-11-08 23:32
</commit_message>
<xml_diff>
--- a/flagged_segments.xlsx
+++ b/flagged_segments.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="39">
   <si>
     <t>Session</t>
   </si>
@@ -34,31 +34,34 @@
     <t>GMT20250821-130122</t>
   </si>
   <si>
+    <t>Yeah, I'm here, but I cannot see you.</t>
+  </si>
+  <si>
+    <t>I'm not able to… My camera doesn't seem to be working.</t>
+  </si>
+  <si>
+    <t>I'm not able to get it to work now.</t>
+  </si>
+  <si>
+    <t>Yeah.</t>
+  </si>
+  <si>
     <t>Hello?</t>
   </si>
   <si>
-    <t>Yeah, I'm here, but I cannot see you.</t>
-  </si>
-  <si>
-    <t>I'm not able to get it to work now.</t>
+    <t>One…</t>
+  </si>
+  <si>
+    <t>There should be…</t>
   </si>
   <si>
     <t>Sorry.</t>
   </si>
   <si>
-    <t>You can try restarting my computer.</t>
-  </si>
-  <si>
-    <t>It's scary, because… If that's how things really work, And we've all been fooled.</t>
-  </si>
-  <si>
-    <t>Yeah, sophomore.</t>
-  </si>
-  <si>
-    <t>We certainly know that religion is being stifled, now, in China.</t>
-  </si>
-  <si>
-    <t>What's that, race called again? The…</t>
+    <t>Where are you?</t>
+  </si>
+  <si>
+    <t>Just try that.</t>
   </si>
   <si>
     <t>Hi, can you hear me?</t>
@@ -73,22 +76,40 @@
     <t>Oh, interesting. I'll double-check my audio, but I think… oh, you can't hear me, one second.</t>
   </si>
   <si>
-    <t>Not, not yet.</t>
-  </si>
-  <si>
-    <t>I am definitely lagging. Or, or I don't know, there's something off.</t>
+    <t>Yeah, I can hear you, Vuz, it's just really delayed.</t>
   </si>
   <si>
     <t>then let me know, I can try my best to…</t>
   </si>
   <si>
-    <t>5 to 10 minutes. I will have to leave by, like, 3 sharp, so I'm really sorry about that. But we can definitely stay on longer next week, because I don't have a meeting right after our session, because usually we meet at 4. Does that work?</t>
-  </si>
-  <si>
-    <t>Hello.</t>
-  </si>
-  <si>
-    <t>I can.</t>
+    <t>….</t>
+  </si>
+  <si>
+    <t>Hello? Oh my god, I'm… I don't know what's happening. …</t>
+  </si>
+  <si>
+    <t>Hello. Oh god.</t>
+  </si>
+  <si>
+    <t>So I can make the….</t>
+  </si>
+  <si>
+    <t>Hello!</t>
+  </si>
+  <si>
+    <t>I can hear you.</t>
+  </si>
+  <si>
+    <t>Gotcha. I think my Wi-Fi should be fine.</t>
+  </si>
+  <si>
+    <t>Does that make sense?</t>
+  </si>
+  <si>
+    <t>Yeah, yeah, now your buck.</t>
+  </si>
+  <si>
+    <t>Hello, can you hear me? I can hear you.</t>
   </si>
   <si>
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20251026-075624_validated_report.html</t>
@@ -97,28 +118,16 @@
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20250821-130122_validated_report.html</t>
   </si>
   <si>
+    <t>Technical: Video Issues</t>
+  </si>
+  <si>
     <t>Technical: Audio Issues</t>
   </si>
   <si>
-    <t>Technical: Video Issues</t>
-  </si>
-  <si>
     <t>Technical: Connectivity Issues</t>
   </si>
   <si>
-    <t>Session Quality: Off-Topic Discussion</t>
-  </si>
-  <si>
     <t>Session Quality: Lack of Engagement</t>
-  </si>
-  <si>
-    <t>Session Quality: Not Understanding the Material</t>
-  </si>
-  <si>
-    <t>Administrative: Payment Adjustments</t>
-  </si>
-  <si>
-    <t>Technical: Screen Sharing Problems</t>
   </si>
   <si>
     <t>View Report</t>
@@ -488,7 +497,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -519,10 +528,10 @@
         <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D2" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -533,10 +542,10 @@
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D3" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -547,10 +556,10 @@
         <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D4" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -561,10 +570,10 @@
         <v>9</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D5" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -572,13 +581,13 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D6" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -586,13 +595,13 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D7" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -600,13 +609,13 @@
         <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -614,13 +623,13 @@
         <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D9" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -628,41 +637,41 @@
         <v>4</v>
       </c>
       <c r="B10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D10" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D11" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D12" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -670,13 +679,13 @@
         <v>5</v>
       </c>
       <c r="B13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D13" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -684,13 +693,13 @@
         <v>5</v>
       </c>
       <c r="B14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D14" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -698,13 +707,13 @@
         <v>5</v>
       </c>
       <c r="B15" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D15" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -712,13 +721,13 @@
         <v>5</v>
       </c>
       <c r="B16" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D16" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -726,13 +735,13 @@
         <v>5</v>
       </c>
       <c r="B17" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D17" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -740,13 +749,13 @@
         <v>5</v>
       </c>
       <c r="B18" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D18" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -754,13 +763,13 @@
         <v>5</v>
       </c>
       <c r="B19" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D19" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -768,13 +777,153 @@
         <v>5</v>
       </c>
       <c r="B20" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D20" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" t="s">
+        <v>5</v>
+      </c>
+      <c r="B21" t="s">
+        <v>23</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D21" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" t="s">
+        <v>5</v>
+      </c>
+      <c r="B22" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D20" t="s">
-        <v>34</v>
+      <c r="C22" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D22" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" t="s">
+        <v>5</v>
+      </c>
+      <c r="B23" t="s">
+        <v>25</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D23" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B24" t="s">
+        <v>22</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D24" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" t="s">
+        <v>5</v>
+      </c>
+      <c r="B25" t="s">
+        <v>26</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D25" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" t="s">
+        <v>5</v>
+      </c>
+      <c r="B26" t="s">
+        <v>27</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D26" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" t="s">
+        <v>5</v>
+      </c>
+      <c r="B27" t="s">
+        <v>28</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D27" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" t="s">
+        <v>5</v>
+      </c>
+      <c r="B28" t="s">
+        <v>29</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D28" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" t="s">
+        <v>5</v>
+      </c>
+      <c r="B29" t="s">
+        <v>30</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D29" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="A30" t="s">
+        <v>5</v>
+      </c>
+      <c r="B30" t="s">
+        <v>31</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D30" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -798,6 +947,16 @@
     <hyperlink ref="C18" r:id="rId17"/>
     <hyperlink ref="C19" r:id="rId18"/>
     <hyperlink ref="C20" r:id="rId19"/>
+    <hyperlink ref="C21" r:id="rId20"/>
+    <hyperlink ref="C22" r:id="rId21"/>
+    <hyperlink ref="C23" r:id="rId22"/>
+    <hyperlink ref="C24" r:id="rId23"/>
+    <hyperlink ref="C25" r:id="rId24"/>
+    <hyperlink ref="C26" r:id="rId25"/>
+    <hyperlink ref="C27" r:id="rId26"/>
+    <hyperlink ref="C28" r:id="rId27"/>
+    <hyperlink ref="C29" r:id="rId28"/>
+    <hyperlink ref="C30" r:id="rId29"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Validated report update 2025-11-08 23:43
</commit_message>
<xml_diff>
--- a/flagged_segments.xlsx
+++ b/flagged_segments.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="43">
   <si>
     <t>Session</t>
   </si>
@@ -40,76 +40,73 @@
     <t>I'm not able to… My camera doesn't seem to be working.</t>
   </si>
   <si>
-    <t>I'm not able to get it to work now.</t>
+    <t>You can try restarting my computer.</t>
+  </si>
+  <si>
+    <t>Woohoo!</t>
+  </si>
+  <si>
+    <t>It's working now.</t>
+  </si>
+  <si>
+    <t>I have no time in my schedule for anything, right?</t>
+  </si>
+  <si>
+    <t>Yeah, so… Yeah, so for a sophomore to get into computer science.</t>
   </si>
   <si>
     <t>Yeah.</t>
   </si>
   <si>
+    <t>So, with the introduction of Sharia law, that was the turning point of the religious tolerance.</t>
+  </si>
+  <si>
+    <t>But with the Columbian Exchange, it was the Northern… pretty much the Northern Europeans turned to rule.</t>
+  </si>
+  <si>
+    <t>… can't… oh, can you hear me?</t>
+  </si>
+  <si>
+    <t>Nope.</t>
+  </si>
+  <si>
+    <t>I can, yeah, but can you hear me?</t>
+  </si>
+  <si>
+    <t>Oh, interesting. I'll double-check my audio, but I think… oh, you can't hear me, one second.</t>
+  </si>
+  <si>
+    <t>Hello? I don't know if you can hear me, but I'll leave the call and just join back.</t>
+  </si>
+  <si>
     <t>Hello?</t>
   </si>
   <si>
-    <t>One…</t>
-  </si>
-  <si>
-    <t>There should be…</t>
-  </si>
-  <si>
-    <t>Sorry.</t>
-  </si>
-  <si>
-    <t>Where are you?</t>
-  </si>
-  <si>
-    <t>Just try that.</t>
-  </si>
-  <si>
-    <t>Hi, can you hear me?</t>
-  </si>
-  <si>
-    <t>… can't… oh, can you hear me?</t>
-  </si>
-  <si>
-    <t>Nope.</t>
-  </si>
-  <si>
-    <t>Oh, interesting. I'll double-check my audio, but I think… oh, you can't hear me, one second.</t>
-  </si>
-  <si>
-    <t>Yeah, I can hear you, Vuz, it's just really delayed.</t>
-  </si>
-  <si>
-    <t>then let me know, I can try my best to…</t>
-  </si>
-  <si>
-    <t>….</t>
+    <t>Gotcha. I think my Wi-Fi should be fine.</t>
+  </si>
+  <si>
+    <t>I am definitely lagging. Or, or I don't know, there's something off.</t>
   </si>
   <si>
     <t>Hello? Oh my god, I'm… I don't know what's happening. …</t>
   </si>
   <si>
+    <t>Is that okay?</t>
+  </si>
+  <si>
     <t>Hello. Oh god.</t>
   </si>
   <si>
-    <t>So I can make the….</t>
-  </si>
-  <si>
-    <t>Hello!</t>
-  </si>
-  <si>
-    <t>I can hear you.</t>
-  </si>
-  <si>
-    <t>Gotcha. I think my Wi-Fi should be fine.</t>
-  </si>
-  <si>
-    <t>Does that make sense?</t>
-  </si>
-  <si>
-    <t>Yeah, yeah, now your buck.</t>
-  </si>
-  <si>
-    <t>Hello, can you hear me? I can hear you.</t>
+    <t>So, what I'm saying is, I'll ask the team to cancel the session from our end.</t>
+  </si>
+  <si>
+    <t>then, we're good, and then I'll make that 30 minutes up for you, and, like, either a free session, or we can just add it to the next session, without you being charged for it.</t>
+  </si>
+  <si>
+    <t>Yeah, but I feel bad just because it wasn't the most efficient 40 minutes. Maybe we can just add a little more time, like, I can stay on for a little longer during our next session, just to kind of make sure that everything we covered today is</t>
+  </si>
+  <si>
+    <t>So…</t>
   </si>
   <si>
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20251026-075624_validated_report.html</t>
@@ -121,13 +118,28 @@
     <t>Technical: Video Issues</t>
   </si>
   <si>
+    <t>Technical: Connectivity Issues</t>
+  </si>
+  <si>
+    <t>Student Behavior Issues: Homework Non-Completion</t>
+  </si>
+  <si>
+    <t>Safety: Inappropriate Language</t>
+  </si>
+  <si>
+    <t>Safety: Illegal Activities</t>
+  </si>
+  <si>
+    <t>Other: Illegal Activities</t>
+  </si>
+  <si>
     <t>Technical: Audio Issues</t>
   </si>
   <si>
-    <t>Technical: Connectivity Issues</t>
-  </si>
-  <si>
-    <t>Session Quality: Lack of Engagement</t>
+    <t>Administrative: Payment Adjustments</t>
+  </si>
+  <si>
+    <t>Administrative: Session Cancellation / Rescheduling</t>
   </si>
   <si>
     <t>View Report</t>
@@ -497,7 +509,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -528,10 +540,10 @@
         <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -542,10 +554,10 @@
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -556,7 +568,7 @@
         <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D4" t="s">
         <v>34</v>
@@ -570,10 +582,10 @@
         <v>9</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -581,13 +593,13 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -595,10 +607,10 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D7" t="s">
         <v>35</v>
@@ -609,13 +621,13 @@
         <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -623,13 +635,13 @@
         <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -637,13 +649,13 @@
         <v>4</v>
       </c>
       <c r="B10" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C10" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D10" t="s">
         <v>38</v>
-      </c>
-      <c r="D10" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -651,27 +663,27 @@
         <v>4</v>
       </c>
       <c r="B11" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D11" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B12" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D12" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -679,13 +691,13 @@
         <v>5</v>
       </c>
       <c r="B13" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D13" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -693,13 +705,13 @@
         <v>5</v>
       </c>
       <c r="B14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D14" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -707,13 +719,13 @@
         <v>5</v>
       </c>
       <c r="B15" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D15" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -721,13 +733,13 @@
         <v>5</v>
       </c>
       <c r="B16" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -735,13 +747,13 @@
         <v>5</v>
       </c>
       <c r="B17" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D17" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -749,13 +761,13 @@
         <v>5</v>
       </c>
       <c r="B18" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D18" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -763,13 +775,13 @@
         <v>5</v>
       </c>
       <c r="B19" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D19" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -777,13 +789,13 @@
         <v>5</v>
       </c>
       <c r="B20" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D20" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -791,13 +803,13 @@
         <v>5</v>
       </c>
       <c r="B21" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D21" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -805,13 +817,13 @@
         <v>5</v>
       </c>
       <c r="B22" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D22" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -819,13 +831,13 @@
         <v>5</v>
       </c>
       <c r="B23" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D23" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -833,13 +845,13 @@
         <v>5</v>
       </c>
       <c r="B24" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D24" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -847,13 +859,13 @@
         <v>5</v>
       </c>
       <c r="B25" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D25" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -861,69 +873,13 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D26" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4">
-      <c r="A27" t="s">
-        <v>5</v>
-      </c>
-      <c r="B27" t="s">
-        <v>28</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D27" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4">
-      <c r="A28" t="s">
-        <v>5</v>
-      </c>
-      <c r="B28" t="s">
-        <v>29</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D28" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4">
-      <c r="A29" t="s">
-        <v>5</v>
-      </c>
-      <c r="B29" t="s">
-        <v>30</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D29" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4">
-      <c r="A30" t="s">
-        <v>5</v>
-      </c>
-      <c r="B30" t="s">
-        <v>31</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D30" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -953,10 +909,6 @@
     <hyperlink ref="C24" r:id="rId23"/>
     <hyperlink ref="C25" r:id="rId24"/>
     <hyperlink ref="C26" r:id="rId25"/>
-    <hyperlink ref="C27" r:id="rId26"/>
-    <hyperlink ref="C28" r:id="rId27"/>
-    <hyperlink ref="C29" r:id="rId28"/>
-    <hyperlink ref="C30" r:id="rId29"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Validated report update 2025-11-09 14:03
</commit_message>
<xml_diff>
--- a/flagged_segments.xlsx
+++ b/flagged_segments.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="44">
   <si>
     <t>Session</t>
   </si>
@@ -34,112 +34,115 @@
     <t>GMT20250821-130122</t>
   </si>
   <si>
+    <t>Ram?</t>
+  </si>
+  <si>
+    <t>Hello?</t>
+  </si>
+  <si>
+    <t>Where are you?</t>
+  </si>
+  <si>
+    <t>One…</t>
+  </si>
+  <si>
+    <t>Hello.</t>
+  </si>
+  <si>
     <t>Yeah, I'm here, but I cannot see you.</t>
   </si>
   <si>
-    <t>I'm not able to… My camera doesn't seem to be working.</t>
-  </si>
-  <si>
-    <t>You can try restarting my computer.</t>
-  </si>
-  <si>
-    <t>Woohoo!</t>
-  </si>
-  <si>
-    <t>It's working now.</t>
-  </si>
-  <si>
-    <t>I have no time in my schedule for anything, right?</t>
-  </si>
-  <si>
-    <t>Yeah, so… Yeah, so for a sophomore to get into computer science.</t>
+    <t>I'm trying to turn on my kit.</t>
+  </si>
+  <si>
+    <t>Okay, I saw you before, so, it…</t>
   </si>
   <si>
     <t>Yeah.</t>
   </si>
   <si>
-    <t>So, with the introduction of Sharia law, that was the turning point of the religious tolerance.</t>
-  </si>
-  <si>
-    <t>But with the Columbian Exchange, it was the Northern… pretty much the Northern Europeans turned to rule.</t>
+    <t>There should be…</t>
+  </si>
+  <si>
+    <t>I'm not able to get it to work now.</t>
+  </si>
+  <si>
+    <t>Hi, can you hear me?</t>
   </si>
   <si>
     <t>… can't… oh, can you hear me?</t>
   </si>
   <si>
+    <t>Hi, how are you? Good to see you!</t>
+  </si>
+  <si>
     <t>Nope.</t>
   </si>
   <si>
+    <t>Hello, can you hear me? I can hear you.</t>
+  </si>
+  <si>
+    <t>Yes, can you hear me?</t>
+  </si>
+  <si>
+    <t>I can hear you.</t>
+  </si>
+  <si>
+    <t>Can you hear me?</t>
+  </si>
+  <si>
     <t>I can, yeah, but can you hear me?</t>
   </si>
   <si>
     <t>Oh, interesting. I'll double-check my audio, but I think… oh, you can't hear me, one second.</t>
   </si>
   <si>
-    <t>Hello? I don't know if you can hear me, but I'll leave the call and just join back.</t>
-  </si>
-  <si>
-    <t>Hello?</t>
-  </si>
-  <si>
-    <t>Gotcha. I think my Wi-Fi should be fine.</t>
-  </si>
-  <si>
-    <t>I am definitely lagging. Or, or I don't know, there's something off.</t>
-  </si>
-  <si>
-    <t>Hello? Oh my god, I'm… I don't know what's happening. …</t>
-  </si>
-  <si>
-    <t>Is that okay?</t>
-  </si>
-  <si>
-    <t>Hello. Oh god.</t>
-  </si>
-  <si>
-    <t>So, what I'm saying is, I'll ask the team to cancel the session from our end.</t>
-  </si>
-  <si>
-    <t>then, we're good, and then I'll make that 30 minutes up for you, and, like, either a free session, or we can just add it to the next session, without you being charged for it.</t>
-  </si>
-  <si>
-    <t>Yeah, but I feel bad just because it wasn't the most efficient 40 minutes. Maybe we can just add a little more time, like, I can stay on for a little longer during our next session, just to kind of make sure that everything we covered today is</t>
-  </si>
-  <si>
-    <t>So…</t>
-  </si>
-  <si>
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20251026-075624_validated_report.html</t>
   </si>
   <si>
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20250821-130122_validated_report.html</t>
   </si>
   <si>
-    <t>Technical: Video Issues</t>
-  </si>
-  <si>
-    <t>Technical: Connectivity Issues</t>
-  </si>
-  <si>
-    <t>Student Behavior Issues: Homework Non-Completion</t>
-  </si>
-  <si>
-    <t>Safety: Inappropriate Language</t>
-  </si>
-  <si>
-    <t>Safety: Illegal Activities</t>
-  </si>
-  <si>
-    <t>Other: Illegal Activities</t>
-  </si>
-  <si>
-    <t>Technical: Audio Issues</t>
-  </si>
-  <si>
-    <t>Administrative: Payment Adjustments</t>
-  </si>
-  <si>
-    <t>Administrative: Session Cancellation / Rescheduling</t>
+    <t>TECHNICAL: audio</t>
+  </si>
+  <si>
+    <t>TECHNICAL: screen share</t>
+  </si>
+  <si>
+    <t>TECHNICAL: lag</t>
+  </si>
+  <si>
+    <t>TECHNICAL: internet</t>
+  </si>
+  <si>
+    <t>POLICY: personal contact info</t>
+  </si>
+  <si>
+    <t>POLICY: grade guarantees</t>
+  </si>
+  <si>
+    <t>BEHAVIOR: homework non-completion</t>
+  </si>
+  <si>
+    <t>QUALITY: tutor doesn't know content</t>
+  </si>
+  <si>
+    <t>QUALITY: lack of engagement</t>
+  </si>
+  <si>
+    <t>SAFETY: profanity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TECHNICAL: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">POLICY: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUALITY: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BEHAVIOR: </t>
   </si>
   <si>
     <t>View Report</t>
@@ -509,7 +512,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -540,10 +543,10 @@
         <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -554,10 +557,10 @@
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D3" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -568,10 +571,10 @@
         <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -582,10 +585,10 @@
         <v>9</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D5" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -596,10 +599,10 @@
         <v>10</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -610,10 +613,10 @@
         <v>11</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -624,10 +627,10 @@
         <v>12</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D8" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -638,10 +641,10 @@
         <v>13</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D9" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -652,10 +655,10 @@
         <v>14</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D10" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -666,24 +669,24 @@
         <v>15</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B12" t="s">
         <v>16</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -694,7 +697,7 @@
         <v>17</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D13" t="s">
         <v>39</v>
@@ -708,7 +711,7 @@
         <v>18</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D14" t="s">
         <v>39</v>
@@ -722,10 +725,10 @@
         <v>19</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D15" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -736,10 +739,10 @@
         <v>20</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D16" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -750,7 +753,7 @@
         <v>21</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D17" t="s">
         <v>39</v>
@@ -761,13 +764,13 @@
         <v>5</v>
       </c>
       <c r="B18" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D18" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -775,13 +778,13 @@
         <v>5</v>
       </c>
       <c r="B19" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D19" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -789,13 +792,13 @@
         <v>5</v>
       </c>
       <c r="B20" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D20" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -803,13 +806,13 @@
         <v>5</v>
       </c>
       <c r="B21" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D21" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -817,13 +820,13 @@
         <v>5</v>
       </c>
       <c r="B22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C22" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D22" t="s">
         <v>42</v>
-      </c>
-      <c r="D22" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -831,55 +834,13 @@
         <v>5</v>
       </c>
       <c r="B23" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C23" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23" t="s">
         <v>42</v>
-      </c>
-      <c r="D23" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4">
-      <c r="A24" t="s">
-        <v>5</v>
-      </c>
-      <c r="B24" t="s">
-        <v>28</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D24" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4">
-      <c r="A25" t="s">
-        <v>5</v>
-      </c>
-      <c r="B25" t="s">
-        <v>29</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D25" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4">
-      <c r="A26" t="s">
-        <v>5</v>
-      </c>
-      <c r="B26" t="s">
-        <v>30</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D26" t="s">
-        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -906,9 +867,6 @@
     <hyperlink ref="C21" r:id="rId20"/>
     <hyperlink ref="C22" r:id="rId21"/>
     <hyperlink ref="C23" r:id="rId22"/>
-    <hyperlink ref="C24" r:id="rId23"/>
-    <hyperlink ref="C25" r:id="rId24"/>
-    <hyperlink ref="C26" r:id="rId25"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Validated report update 2025-11-09 17:21
</commit_message>
<xml_diff>
--- a/flagged_segments.xlsx
+++ b/flagged_segments.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="32">
   <si>
     <t>Session</t>
   </si>
@@ -34,37 +34,34 @@
     <t>GMT20250821-130122</t>
   </si>
   <si>
-    <t>Ram?</t>
-  </si>
-  <si>
     <t>Hello?</t>
   </si>
   <si>
-    <t>Where are you?</t>
-  </si>
-  <si>
-    <t>One…</t>
-  </si>
-  <si>
-    <t>Hello.</t>
-  </si>
-  <si>
     <t>Yeah, I'm here, but I cannot see you.</t>
   </si>
   <si>
-    <t>I'm trying to turn on my kit.</t>
-  </si>
-  <si>
-    <t>Okay, I saw you before, so, it…</t>
+    <t>I'm not able to get it to work now.</t>
+  </si>
+  <si>
+    <t>I'm not able to… My camera doesn't seem to be working.</t>
+  </si>
+  <si>
+    <t>Yes, it can often fix it.</t>
+  </si>
+  <si>
+    <t>I mean, on Tuesday, so…</t>
   </si>
   <si>
     <t>Yeah.</t>
   </si>
   <si>
-    <t>There should be…</t>
-  </si>
-  <si>
-    <t>I'm not able to get it to work now.</t>
+    <t>Hmm.</t>
+  </si>
+  <si>
+    <t>I think some of them were in the Ottoman Empire, were soldiers, and were called Janissaries, but…</t>
+  </si>
+  <si>
+    <t>So, for us to romanticize any of these time periods, we would be foolhardy to think so.</t>
   </si>
   <si>
     <t>Hi, can you hear me?</t>
@@ -73,76 +70,43 @@
     <t>… can't… oh, can you hear me?</t>
   </si>
   <si>
-    <t>Hi, how are you? Good to see you!</t>
-  </si>
-  <si>
     <t>Nope.</t>
   </si>
   <si>
-    <t>Hello, can you hear me? I can hear you.</t>
-  </si>
-  <si>
-    <t>Yes, can you hear me?</t>
-  </si>
-  <si>
-    <t>I can hear you.</t>
-  </si>
-  <si>
-    <t>Can you hear me?</t>
-  </si>
-  <si>
-    <t>I can, yeah, but can you hear me?</t>
-  </si>
-  <si>
     <t>Oh, interesting. I'll double-check my audio, but I think… oh, you can't hear me, one second.</t>
   </si>
   <si>
+    <t>Yeah, I can hear you, Vuz, it's just really delayed.</t>
+  </si>
+  <si>
+    <t>Gotcha. I think my Wi-Fi should be fine.</t>
+  </si>
+  <si>
+    <t>I am definitely lagging. Or, or I don't know, there's something off.</t>
+  </si>
+  <si>
+    <t>Wi-Fi or yours. Give me just a second, I'll try to restart my Wi-Fi very quickly.</t>
+  </si>
+  <si>
+    <t>Okay, can you hear me now?</t>
+  </si>
+  <si>
+    <t>It's unfair to you if we just go on like this for the next 30, 40 minutes of this session. If the internet issue continues happening, then I'll just ask them to, like, not charge you for the session. Hello? Can you hear me?</t>
+  </si>
+  <si>
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20251026-075624_validated_report.html</t>
   </si>
   <si>
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20250821-130122_validated_report.html</t>
   </si>
   <si>
-    <t>TECHNICAL: audio</t>
-  </si>
-  <si>
-    <t>TECHNICAL: screen share</t>
-  </si>
-  <si>
-    <t>TECHNICAL: lag</t>
-  </si>
-  <si>
-    <t>TECHNICAL: internet</t>
-  </si>
-  <si>
-    <t>POLICY: personal contact info</t>
-  </si>
-  <si>
-    <t>POLICY: grade guarantees</t>
-  </si>
-  <si>
-    <t>BEHAVIOR: homework non-completion</t>
-  </si>
-  <si>
-    <t>QUALITY: tutor doesn't know content</t>
-  </si>
-  <si>
-    <t>QUALITY: lack of engagement</t>
-  </si>
-  <si>
-    <t>SAFETY: profanity</t>
-  </si>
-  <si>
     <t xml:space="preserve">TECHNICAL: </t>
   </si>
   <si>
-    <t xml:space="preserve">POLICY: </t>
-  </si>
-  <si>
     <t xml:space="preserve">QUALITY: </t>
   </si>
   <si>
-    <t xml:space="preserve">BEHAVIOR: </t>
+    <t xml:space="preserve">ADMIN: </t>
   </si>
   <si>
     <t>View Report</t>
@@ -512,7 +476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -543,10 +507,10 @@
         <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -557,10 +521,10 @@
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -571,10 +535,10 @@
         <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D4" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -585,10 +549,10 @@
         <v>9</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -599,10 +563,10 @@
         <v>10</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D6" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -613,10 +577,10 @@
         <v>11</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D7" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -627,10 +591,10 @@
         <v>12</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D8" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -641,10 +605,10 @@
         <v>13</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D9" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -655,10 +619,10 @@
         <v>14</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D10" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -669,24 +633,24 @@
         <v>15</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D11" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B12" t="s">
         <v>16</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D12" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -697,10 +661,10 @@
         <v>17</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D13" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -711,10 +675,10 @@
         <v>18</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D14" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -725,10 +689,10 @@
         <v>19</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D15" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -739,10 +703,10 @@
         <v>20</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D16" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -753,10 +717,10 @@
         <v>21</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D17" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -764,13 +728,13 @@
         <v>5</v>
       </c>
       <c r="B18" t="s">
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D18" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -778,13 +742,13 @@
         <v>5</v>
       </c>
       <c r="B19" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D19" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -792,13 +756,13 @@
         <v>5</v>
       </c>
       <c r="B20" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D20" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -806,41 +770,13 @@
         <v>5</v>
       </c>
       <c r="B21" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D21" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4">
-      <c r="A22" t="s">
-        <v>5</v>
-      </c>
-      <c r="B22" t="s">
-        <v>25</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D22" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4">
-      <c r="A23" t="s">
-        <v>5</v>
-      </c>
-      <c r="B23" t="s">
-        <v>26</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D23" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -865,8 +801,6 @@
     <hyperlink ref="C19" r:id="rId18"/>
     <hyperlink ref="C20" r:id="rId19"/>
     <hyperlink ref="C21" r:id="rId20"/>
-    <hyperlink ref="C22" r:id="rId21"/>
-    <hyperlink ref="C23" r:id="rId22"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Validated report update 2025-11-09 17:32
</commit_message>
<xml_diff>
--- a/flagged_segments.xlsx
+++ b/flagged_segments.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="37">
   <si>
     <t>Session</t>
   </si>
@@ -37,31 +37,43 @@
     <t>Hello?</t>
   </si>
   <si>
+    <t>Hello.</t>
+  </si>
+  <si>
+    <t>I'm not able to… My camera doesn't seem to be working.</t>
+  </si>
+  <si>
     <t>Yeah, I'm here, but I cannot see you.</t>
   </si>
   <si>
     <t>I'm not able to get it to work now.</t>
   </si>
   <si>
-    <t>I'm not able to… My camera doesn't seem to be working.</t>
+    <t>I'm trying to turn on my kit.</t>
+  </si>
+  <si>
+    <t>It's working now.</t>
   </si>
   <si>
     <t>Yes, it can often fix it.</t>
   </si>
   <si>
-    <t>I mean, on Tuesday, so…</t>
-  </si>
-  <si>
-    <t>Yeah.</t>
-  </si>
-  <si>
-    <t>Hmm.</t>
-  </si>
-  <si>
-    <t>I think some of them were in the Ottoman Empire, were soldiers, and were called Janissaries, but…</t>
-  </si>
-  <si>
-    <t>So, for us to romanticize any of these time periods, we would be foolhardy to think so.</t>
+    <t>One…</t>
+  </si>
+  <si>
+    <t>In school.</t>
+  </si>
+  <si>
+    <t>Because there are an awful lot of countries in the world, and you have a… you have a good sense of when the book talks about.</t>
+  </si>
+  <si>
+    <t>Yeah, keep going.</t>
+  </si>
+  <si>
+    <t>for what's going on, you're just trying to get all of this information stuffed into your head so you can make sense of something. But without having some context, it makes it quite difficult to put all the pieces together.</t>
+  </si>
+  <si>
+    <t>Now we have a communist government that literally controls… everything.</t>
   </si>
   <si>
     <t>Hi, can you hear me?</t>
@@ -70,9 +82,6 @@
     <t>… can't… oh, can you hear me?</t>
   </si>
   <si>
-    <t>Nope.</t>
-  </si>
-  <si>
     <t>Oh, interesting. I'll double-check my audio, but I think… oh, you can't hear me, one second.</t>
   </si>
   <si>
@@ -85,13 +94,16 @@
     <t>I am definitely lagging. Or, or I don't know, there's something off.</t>
   </si>
   <si>
-    <t>Wi-Fi or yours. Give me just a second, I'll try to restart my Wi-Fi very quickly.</t>
-  </si>
-  <si>
-    <t>Okay, can you hear me now?</t>
-  </si>
-  <si>
-    <t>It's unfair to you if we just go on like this for the next 30, 40 minutes of this session. If the internet issue continues happening, then I'll just ask them to, like, not charge you for the session. Hello? Can you hear me?</t>
+    <t>Hello. Oh god.</t>
+  </si>
+  <si>
+    <t>then, we're good, and then I'll make that 30 minutes up for you, and, like, either a free session, or we can just add it to the next session, without you being charged for it.</t>
+  </si>
+  <si>
+    <t>I can't cue you.</t>
+  </si>
+  <si>
+    <t>Is that fine? I think it's just unfair to you that I just talk and you spend, like, half the time deciphering what I'm saying because of internet issues.</t>
   </si>
   <si>
     <t>https://andreamaria810.github.io/Zoom_Reports/html_reports/GMT20251026-075624_validated_report.html</t>
@@ -101,6 +113,9 @@
   </si>
   <si>
     <t xml:space="preserve">TECHNICAL: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BEHAVIOR: </t>
   </si>
   <si>
     <t xml:space="preserve">QUALITY: </t>
@@ -476,7 +491,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -507,10 +522,10 @@
         <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -521,10 +536,10 @@
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D3" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -535,10 +550,10 @@
         <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -549,10 +564,10 @@
         <v>9</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D5" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -560,13 +575,13 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -574,13 +589,13 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -588,13 +603,13 @@
         <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D8" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -602,13 +617,13 @@
         <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D9" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -616,13 +631,13 @@
         <v>4</v>
       </c>
       <c r="B10" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D10" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -630,111 +645,111 @@
         <v>4</v>
       </c>
       <c r="B11" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D11" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B12" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D12" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B13" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D13" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B14" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D14" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B15" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D15" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B16" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D16" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B17" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D17" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B18" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D18" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -742,13 +757,13 @@
         <v>5</v>
       </c>
       <c r="B19" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D19" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -756,13 +771,13 @@
         <v>5</v>
       </c>
       <c r="B20" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D20" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -770,13 +785,111 @@
         <v>5</v>
       </c>
       <c r="B21" t="s">
+        <v>22</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D21" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" t="s">
+        <v>5</v>
+      </c>
+      <c r="B22" t="s">
+        <v>23</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D22" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" t="s">
+        <v>5</v>
+      </c>
+      <c r="B23" t="s">
+        <v>24</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D23" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B24" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D21" t="s">
-        <v>30</v>
+      <c r="C24" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D24" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" t="s">
+        <v>5</v>
+      </c>
+      <c r="B25" t="s">
+        <v>26</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D25" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" t="s">
+        <v>5</v>
+      </c>
+      <c r="B26" t="s">
+        <v>27</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D26" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" t="s">
+        <v>5</v>
+      </c>
+      <c r="B27" t="s">
+        <v>28</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D27" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" t="s">
+        <v>5</v>
+      </c>
+      <c r="B28" t="s">
+        <v>29</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D28" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -801,6 +914,13 @@
     <hyperlink ref="C19" r:id="rId18"/>
     <hyperlink ref="C20" r:id="rId19"/>
     <hyperlink ref="C21" r:id="rId20"/>
+    <hyperlink ref="C22" r:id="rId21"/>
+    <hyperlink ref="C23" r:id="rId22"/>
+    <hyperlink ref="C24" r:id="rId23"/>
+    <hyperlink ref="C25" r:id="rId24"/>
+    <hyperlink ref="C26" r:id="rId25"/>
+    <hyperlink ref="C27" r:id="rId26"/>
+    <hyperlink ref="C28" r:id="rId27"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>